<commit_message>
📊 Horarios actualizados Línea 141 - 4298
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:28:37</t>
+          <t>Última actualización: 01:07:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>00:28:37</t>
+          <t>01:07:01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -487,9 +487,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>57</v>
+        <v>18</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>01:07:01</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>03:02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>115</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -519,7 +544,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:28:37</t>
+          <t>Última actualización: 01:07:01</t>
         </is>
       </c>
     </row>
@@ -554,7 +579,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:28:37</t>
+          <t>Última actualización: 01:07:01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4299
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:07:01</t>
+          <t>Última actualización: 01:45:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 1</t>
         </is>
       </c>
     </row>
@@ -473,48 +473,23 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:07:01</t>
+          <t>01:45:46</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:25</t>
+          <t>03:01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="E6" t="inlineStr">
-        <is>
-          <t>LP1912</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>01:07:01</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>03:02</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>15_ABASTO</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>115</v>
-      </c>
-      <c r="E7" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -544,7 +519,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:07:01</t>
+          <t>Última actualización: 01:45:46</t>
         </is>
       </c>
     </row>
@@ -579,7 +554,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:07:01</t>
+          <t>Última actualización: 01:45:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4300
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:45:46</t>
+          <t>Última actualización: 02:08:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:45:46</t>
+          <t>02:08:32</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -487,9 +487,59 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>02:08:32</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>03:48</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:08:32</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>04:02</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>114</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -519,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:45:46</t>
+          <t>Última actualización: 02:08:32</t>
         </is>
       </c>
     </row>
@@ -554,7 +604,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:45:46</t>
+          <t>Última actualización: 02:08:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4301
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:08:32</t>
+          <t>Última actualización: 02:38:03</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:08:32</t>
+          <t>02:38:02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:01</t>
+          <t>03:02</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,7 +498,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:08:32</t>
+          <t>02:38:02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,7 +523,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:08:32</t>
+          <t>02:38:02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:08:32</t>
+          <t>Última actualización: 02:38:03</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:08:32</t>
+          <t>Última actualización: 02:38:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4302
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:38:03</t>
+          <t>Última actualización: 02:57:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:38:02</t>
+          <t>02:57:39</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>03:01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,7 +498,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:38:02</t>
+          <t>02:57:39</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,7 +523,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:38:02</t>
+          <t>02:57:39</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -537,9 +537,59 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>02:57:39</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:47</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>110</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>02:57:39</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>04:53</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>116</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -569,7 +619,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:38:03</t>
+          <t>Última actualización: 02:57:39</t>
         </is>
       </c>
     </row>
@@ -604,7 +654,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:38:03</t>
+          <t>Última actualización: 02:57:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4303
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:57:39</t>
+          <t>Última actualización: 03:29:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:57:39</t>
+          <t>03:29:22</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:01</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:57:39</t>
+          <t>03:29:22</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,12 +523,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:57:39</t>
+          <t>03:29:22</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:02</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>02:57:39</t>
+          <t>03:29:22</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>110</v>
+        <v>84</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,23 +573,48 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>02:57:39</t>
+          <t>03:29:22</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>03:29:22</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:22</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>113</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -619,7 +644,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:57:39</t>
+          <t>Última actualización: 03:29:22</t>
         </is>
       </c>
     </row>
@@ -654,7 +679,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:57:39</t>
+          <t>Última actualización: 03:29:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4304
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:29:22</t>
+          <t>Última actualización: 04:08:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:29:22</t>
+          <t>04:08:49</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:29:22</t>
+          <t>04:08:49</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:02</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:29:22</t>
+          <t>04:08:49</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>05:16</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:29:22</t>
+          <t>04:08:49</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:29:22</t>
+          <t>04:08:49</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>05:46</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,23 +598,48 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:29:22</t>
+          <t>04:08:49</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:56</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
+        <v>108</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>04:08:49</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
         <v>113</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -644,7 +669,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:29:22</t>
+          <t>Última actualización: 04:08:49</t>
         </is>
       </c>
     </row>
@@ -679,7 +704,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:29:22</t>
+          <t>Última actualización: 04:08:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4305
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:08:49</t>
+          <t>Última actualización: 04:40:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:08:49</t>
+          <t>04:40:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,7 +498,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:08:49</t>
+          <t>04:40:40</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,12 +523,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:08:49</t>
+          <t>04:40:40</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:16</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,7 +548,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:08:49</t>
+          <t>04:40:40</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:08:49</t>
+          <t>04:40:40</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:46</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>98</v>
+        <v>64</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:08:49</t>
+          <t>04:40:40</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:56</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>108</v>
+        <v>67</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,7 +623,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:08:49</t>
+          <t>04:40:40</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -637,9 +637,134 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:40:40</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:09</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>89</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:40:40</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>92</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:40:40</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>110</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:40:40</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:36</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>116</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:40:40</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>119</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -656,7 +781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -669,14 +794,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:08:49</t>
+          <t>Última actualización: 04:40:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>04:40:40</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>92</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -704,7 +881,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:08:49</t>
+          <t>Última actualización: 04:40:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4306
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:40:40</t>
+          <t>Última actualización: 05:00:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:40:40</t>
+          <t>05:00:42</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>05:16</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:40:40</t>
+          <t>05:00:42</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:40:40</t>
+          <t>05:00:42</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:40:40</t>
+          <t>05:00:42</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:46</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:40:40</t>
+          <t>05:00:42</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:40:40</t>
+          <t>05:00:42</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:40:40</t>
+          <t>05:00:42</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:40:40</t>
+          <t>05:00:42</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:40:40</t>
+          <t>05:00:42</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:36</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:40:40</t>
+          <t>05:00:42</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:40:40</t>
+          <t>05:00:42</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,23 +748,48 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:40:40</t>
+          <t>05:00:42</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D17" t="n">
+        <v>101</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>05:00:42</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:59</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
         <v>119</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -794,7 +819,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:40:40</t>
+          <t>Última actualización: 05:00:42</t>
         </is>
       </c>
     </row>
@@ -835,7 +860,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:40:40</t>
+          <t>05:00:42</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -849,7 +874,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -881,7 +906,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:40:40</t>
+          <t>Última actualización: 05:00:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4307
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:00:42</t>
+          <t>Última actualización: 05:40:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:00:42</t>
+          <t>05:40:39</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:16</t>
+          <t>05:42</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:00:42</t>
+          <t>05:40:39</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:00:42</t>
+          <t>05:40:39</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:00:42</t>
+          <t>05:40:39</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:46</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:00:42</t>
+          <t>05:40:39</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:00:42</t>
+          <t>05:40:39</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:36</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:00:42</t>
+          <t>05:40:39</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:00:42</t>
+          <t>05:40:39</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:00:42</t>
+          <t>05:40:39</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>96</v>
+        <v>61</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:00:42</t>
+          <t>05:40:39</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:00:42</t>
+          <t>05:40:39</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:00:42</t>
+          <t>05:40:39</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,23 +773,123 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:00:42</t>
+          <t>05:40:39</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>05:40:39</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07:27</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>107</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>05:40:39</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>111</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>05:40:39</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>116</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>05:40:39</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>07:38</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>118</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -806,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -819,14 +919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:00:42</t>
+          <t>Última actualización: 05:40:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -860,7 +960,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:00:42</t>
+          <t>05:40:39</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -874,9 +974,59 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:40:39</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>82</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>05:40:39</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>111</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -906,7 +1056,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:00:42</t>
+          <t>Última actualización: 05:40:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4308
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:40:39</t>
+          <t>Última actualización: 06:03:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:42</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:36</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:41</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,48 +848,23 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="E21" t="inlineStr">
-        <is>
-          <t>LP1912</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>05:40:39</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>07:38</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>14_ABASTO</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>118</v>
-      </c>
-      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -919,7 +894,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:40:39</t>
+          <t>Última actualización: 06:03:22</t>
         </is>
       </c>
     </row>
@@ -960,7 +935,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -974,7 +949,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -985,7 +960,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -999,7 +974,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1010,12 +985,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:40:39</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1024,7 +999,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1043,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1056,14 +1031,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:40:39</t>
+          <t>Última actualización: 06:03:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06:03:22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>106</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4309
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:03:22</t>
+          <t>Última actualización: 06:35:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:35:47</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:38</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:35:47</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:35:47</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:35:47</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>56</v>
+        <v>5</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -678,16 +678,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:35:47</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:35:47</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:35:47</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -803,16 +803,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,12 +823,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:35:47</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:41</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -837,7 +837,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>98</v>
+        <v>51</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -853,18 +853,343 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>07:26</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>83</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>06:35:47</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>07:28</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>53</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>06:35:47</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>07:29</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>54</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>06:03:22</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>87</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>06:35:47</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>56</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>06:03:22</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>89</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>06:35:47</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>61</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>06:03:22</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>94</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>06:03:22</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>07:41</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>98</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>06:35:47</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>07:44</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>101</v>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="D30" t="n">
+        <v>69</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>06:35:47</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>76</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>06:35:47</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>104</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>06:35:47</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>106</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>06:35:47</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>08:25</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>110</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -881,7 +1206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -894,14 +1219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:03:22</t>
+          <t>Última actualización: 06:35:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -960,7 +1285,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:35:47</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -974,7 +1299,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -985,23 +1310,73 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>06:35:47</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>56</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>06:03:22</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>07:32</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D9" t="n">
         <v>89</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06:35:47</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>76</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1018,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1031,14 +1406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:03:22</t>
+          <t>Última actualización: 06:35:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -1072,23 +1447,48 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>06:35:47</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>73</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>06:03:22</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>07:49</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D7" t="n">
         <v>106</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4310
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:35:47</t>
+          <t>Última actualización: 06:53:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -723,12 +723,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>06:58</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -753,16 +753,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,12 +798,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>78</v>
+        <v>27</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>83</v>
+        <v>33</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,21 +873,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -903,16 +903,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,12 +923,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:35:47</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>87</v>
+        <v>54</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,21 +948,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,12 +973,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>89</v>
+        <v>38</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,12 +1023,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>94</v>
+        <v>43</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1053,16 +1053,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>07:41</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:41</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>07:51</t>
+          <t>07:43</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1128,16 +1128,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>07:46</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>106</v>
+        <v>53</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,23 +1173,173 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>58</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>06:53:53</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>67</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>06:53:53</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>86</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>06:53:53</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>88</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>06:53:53</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>08:25</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>110</v>
-      </c>
-      <c r="E34" t="inlineStr">
+      <c r="D38" t="n">
+        <v>92</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>06:53:53</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>111</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>06:53:53</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>111</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1206,7 +1356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1219,14 +1369,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:35:47</t>
+          <t>Última actualización: 06:53:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1435,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1299,7 +1449,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1310,7 +1460,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1324,7 +1474,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1360,7 +1510,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1374,9 +1524,59 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:53:53</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>111</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>06:53:53</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>111</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1393,7 +1593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1406,14 +1606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:35:47</t>
+          <t>Última actualización: 06:53:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1647,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1461,7 +1661,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1489,6 +1689,31 @@
         <v>106</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:53:53</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>104</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4311
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:53:53</t>
+          <t>Última actualización: 07:10:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -858,7 +858,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -883,11 +883,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -928,16 +928,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,12 +948,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>06:35:47</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>87</v>
+        <v>54</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,21 +973,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>38</v>
+        <v>87</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,12 +998,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,12 +1048,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1078,16 +1078,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>07:41</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>06:03:22</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>07:43</t>
+          <t>07:41</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,12 +1123,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:35:47</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:43</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,12 +1148,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>07:46</t>
+          <t>07:43</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>07:51</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1203,16 +1203,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:46</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,21 +1223,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>86</v>
+        <v>41</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1253,16 +1253,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>08:25</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>111</v>
+        <v>69</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,23 +1323,148 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>71</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>07:10:45</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>08:25</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>75</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>07:10:45</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>08:44</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>94</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>07:10:45</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D40" t="n">
-        <v>111</v>
-      </c>
-      <c r="E40" t="inlineStr">
+      <c r="D43" t="n">
+        <v>94</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>07:10:45</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>114</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>07:10:45</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>116</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1356,7 +1481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1369,14 +1494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:53:53</t>
+          <t>Última actualización: 07:10:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1585,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1474,7 +1599,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1510,7 +1635,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1524,7 +1649,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1535,7 +1660,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1549,7 +1674,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>111</v>
+        <v>94</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1560,7 +1685,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1574,9 +1699,34 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>111</v>
+        <v>94</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07:10:45</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>116</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1593,7 +1743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1606,14 +1756,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:53:53</t>
+          <t>Última actualización: 07:10:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1797,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1661,7 +1811,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1697,7 +1847,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1711,11 +1861,36 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:10:45</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>112</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4312
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:10:45</t>
+          <t>Última actualización: 07:40:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -883,11 +883,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:40:10</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1223,7 +1223,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:40:10</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:40:10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:40:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>69</v>
+        <v>26</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:40:10</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:40:10</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>08:25</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>75</v>
+        <v>41</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1378,16 +1378,16 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:25</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:40:10</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:26</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>94</v>
+        <v>46</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1428,16 +1428,16 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1453,18 +1453,268 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>94</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>07:40:10</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>65</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>07:40:10</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>65</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>07:40:10</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>84</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>07:40:10</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>09:06</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D45" t="n">
-        <v>116</v>
-      </c>
-      <c r="E45" t="inlineStr">
+      <c r="D49" t="n">
+        <v>86</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>07:40:10</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>91</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>07:40:10</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>96</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>07:40:10</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>97</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>07:40:10</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>104</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>07:40:10</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>114</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>07:40:10</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>115</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1481,7 +1731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1494,14 +1744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:10:45</t>
+          <t>Última actualización: 07:40:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1635,7 +1885,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:40:10</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1649,7 +1899,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1710,23 +1960,73 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:40:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>65</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07:40:10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>65</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>07:40:10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>09:06</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>116</v>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D15" t="n">
+        <v>86</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1743,7 +2043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1756,14 +2056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:10:45</t>
+          <t>Última actualización: 07:40:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1822,7 +2122,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:03:22</t>
+          <t>07:40:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1836,7 +2136,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>106</v>
+        <v>9</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1872,23 +2172,73 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>07:40:10</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>58</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>07:10:45</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>09:02</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D10" t="n">
         <v>112</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07:40:10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>83</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4313
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:40:10</t>
+          <t>Última actualización: 07:55:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 50</t>
+          <t>Total filas: 54</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -883,11 +883,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1362,7 +1362,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>94</v>
+        <v>46</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>94</v>
+        <v>49</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,12 +1473,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1528,16 +1528,16 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>91</v>
+        <v>71</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:08</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1628,16 +1628,16 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>104</v>
+        <v>81</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1678,16 +1678,16 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>114</v>
+        <v>96</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1703,18 +1703,118 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>97</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>89</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>99</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
           <t>09:35</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D55" t="n">
-        <v>115</v>
-      </c>
-      <c r="E55" t="inlineStr">
+      <c r="D58" t="n">
+        <v>100</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>109</v>
+      </c>
+      <c r="E59" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1744,7 +1844,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:40:10</t>
+          <t>Última actualización: 07:55:48</t>
         </is>
       </c>
     </row>
@@ -1910,7 +2010,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1924,7 +2024,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>94</v>
+        <v>49</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1935,7 +2035,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1949,7 +2049,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>94</v>
+        <v>49</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2010,7 +2110,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2024,7 +2124,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2043,7 +2143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2056,14 +2156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:40:10</t>
+          <t>Última actualización: 07:55:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2247,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2161,7 +2261,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>87</v>
+        <v>42</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2197,7 +2297,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2211,7 +2311,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>112</v>
+        <v>67</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2241,6 +2341,31 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>92</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4314
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:55:48</t>
+          <t>Última actualización: 08:10:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 54</t>
+          <t>Total filas: 60</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>08:25</t>
+          <t>08:22</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,12 +1398,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>08:26</t>
+          <t>08:25</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:26</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1603,16 +1603,16 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>09:08</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,12 +1623,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>91</v>
+        <v>57</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:08</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1703,16 +1703,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1753,16 +1753,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>07:40:10</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,23 +1798,173 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>08:10:01</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>74</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>08:10:01</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>84</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>08:10:01</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>85</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>07:55:48</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>09:44</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D59" t="n">
+      <c r="D62" t="n">
         <v>109</v>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>08:10:01</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>95</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>08:10:01</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>105</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>08:10:01</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>117</v>
+      </c>
+      <c r="E65" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1831,7 +1981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1844,14 +1994,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:55:48</t>
+          <t>Última actualización: 08:10:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2060,7 +2210,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2074,7 +2224,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2085,7 +2235,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2099,7 +2249,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2127,6 +2277,56 @@
         <v>71</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:10:01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>57</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:10:01</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>105</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2143,7 +2343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2156,14 +2356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:55:48</t>
+          <t>Última actualización: 08:10:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2472,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2286,7 +2486,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2322,7 +2522,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2336,7 +2536,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>83</v>
+        <v>53</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2364,6 +2564,31 @@
         <v>92</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:10:01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>78</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4315
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:10:01</t>
+          <t>Última actualización: 08:31:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 60</t>
+          <t>Total filas: 65</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -883,11 +883,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1462,7 +1462,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1512,7 +1512,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1587,7 +1587,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>91</v>
+        <v>40</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>81</v>
+        <v>45</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1812,7 +1812,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>109</v>
+        <v>73</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1923,12 +1923,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>105</v>
+        <v>83</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1953,18 +1953,143 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>105</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>08:31:38</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>09:59</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>88</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>08:31:38</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>93</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>08:10:01</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
           <t>10:07</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D65" t="n">
+      <c r="D68" t="n">
         <v>117</v>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>08:31:38</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>104</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>08:31:38</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>113</v>
+      </c>
+      <c r="E70" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1981,7 +2106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1994,14 +2119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:10:01</t>
+          <t>Última actualización: 08:31:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2285,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2174,7 +2299,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2185,7 +2310,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2199,7 +2324,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2260,7 +2385,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2274,7 +2399,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2310,23 +2435,48 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>08:31:38</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>83</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>08:10:01</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>09:55</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D18" t="n">
         <v>105</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2343,7 +2493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2356,14 +2506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:10:01</t>
+          <t>Última actualización: 08:31:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -2447,7 +2597,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2461,7 +2611,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2497,7 +2647,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2511,7 +2661,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>67</v>
+        <v>31</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2547,7 +2697,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2561,7 +2711,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>92</v>
+        <v>56</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2589,6 +2739,56 @@
         <v>78</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:31:38</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10:17</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>106</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:31:38</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>119</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4316
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:31:38</t>
+          <t>Última actualización: 08:50:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 65</t>
+          <t>Total filas: 70</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -883,11 +883,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1587,7 +1587,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1812,7 +1812,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>09:54</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>83</v>
+        <v>61</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:52</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>105</v>
+        <v>62</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>09:59</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>10:07</t>
+          <t>09:57</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>117</v>
+        <v>67</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2053,16 +2053,16 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>09:59</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,23 +2073,148 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>74</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>08:10:01</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>117</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>08:50:45</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>85</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>08:50:45</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t>10:24</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D70" t="n">
-        <v>113</v>
-      </c>
-      <c r="E70" t="inlineStr">
+      <c r="D73" t="n">
+        <v>94</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>08:50:45</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>104</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>08:50:45</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>114</v>
+      </c>
+      <c r="E75" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2119,7 +2244,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:31:38</t>
+          <t>Última actualización: 08:50:45</t>
         </is>
       </c>
     </row>
@@ -2385,7 +2510,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2399,7 +2524,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2435,7 +2560,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2449,7 +2574,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2493,7 +2618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2506,14 +2631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:31:38</t>
+          <t>Última actualización: 08:50:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2772,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2661,7 +2786,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2697,7 +2822,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2711,7 +2836,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2747,7 +2872,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2761,7 +2886,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2772,23 +2897,73 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>08:50:45</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>99</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>08:31:38</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D16" t="n">
         <v>119</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:50:45</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>112</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4317
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:50:45</t>
+          <t>Última actualización: 09:14:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 70</t>
+          <t>Total filas: 77</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -883,11 +883,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:14</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:40:10</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>97</v>
+        <v>2</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>07:40:10</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:35</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,12 +1898,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>95</v>
+        <v>30</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>61</v>
+        <v>95</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>09:52</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>62</v>
+        <v>37</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1978,16 +1978,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>09:54</t>
+          <t>09:52</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,12 +1998,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>105</v>
+        <v>64</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,12 +2048,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>09:59</t>
+          <t>09:57</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>08:31:38</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>09:59</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>10:07</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>117</v>
+        <v>47</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:07</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:14</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>104</v>
+        <v>60</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,23 +2198,198 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>61</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>09:14:25</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>70</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>09:14:25</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>80</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>09:14:25</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
           <t>10:44</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D75" t="n">
+      <c r="D78" t="n">
+        <v>90</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>09:14:25</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>101</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>09:14:25</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>102</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>09:14:25</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>110</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>09:14:25</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
         <v>114</v>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="E82" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2244,7 +2419,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:50:45</t>
+          <t>Última actualización: 09:14:25</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2760,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2599,7 +2774,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>105</v>
+        <v>41</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2618,7 +2793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2631,14 +2806,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:50:45</t>
+          <t>Última actualización: 09:14:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2847,7 +3022,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2861,7 +3036,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>78</v>
+        <v>14</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2897,37 +3072,37 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10:29</t>
+          <t>10:18</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:31:38</t>
+          <t>08:50:45</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:29</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2936,7 +3111,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2947,23 +3122,73 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>09:14:25</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>76</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>08:50:45</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>10:42</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D18" t="n">
         <v>112</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>09:14:25</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>89</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4318
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:14:25</t>
+          <t>Última actualización: 10:00:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 77</t>
+          <t>Total filas: 91</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2123,12 +2123,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>09:14:25</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>10:03</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,12 +2148,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:10:01</t>
+          <t>09:14:25</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>10:07</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2162,7 +2162,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>117</v>
+        <v>50</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>09:14:25</t>
+          <t>08:10:01</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>10:14</t>
+          <t>10:07</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>60</v>
+        <v>117</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2203,16 +2203,16 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>10:14</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>09:14:25</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>09:14:25</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:24</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>80</v>
+        <v>24</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,21 +2273,21 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>09:14:25</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>90</v>
+        <v>26</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>09:14:25</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:34</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,12 +2323,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>09:14:25</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>10:56</t>
+          <t>10:41</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2337,7 +2337,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>102</v>
+        <v>41</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>09:14:25</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>110</v>
+        <v>43</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2378,18 +2378,368 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>90</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>51</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>55</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>09:14:25</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>102</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>64</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>11:07</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>67</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>09:14:25</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
           <t>11:08</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>225_C ROCA-H SUR</t>
         </is>
       </c>
-      <c r="D82" t="n">
+      <c r="D88" t="n">
         <v>114</v>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>11:12</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>72</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>83</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>94</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>95</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>11:37</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>97</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>104</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>114</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>115</v>
+      </c>
+      <c r="E96" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2406,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2419,14 +2769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:14:25</t>
+          <t>Última actualización: 10:00:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2777,6 +3127,56 @@
         <v>41</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>94</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>104</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2793,7 +3193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2806,14 +3206,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:14:25</t>
+          <t>Última actualización: 10:00:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -3047,7 +3447,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3061,7 +3461,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>87</v>
+        <v>17</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -3097,7 +3497,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3111,7 +3511,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>99</v>
+        <v>29</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3147,7 +3547,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:50:45</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3161,7 +3561,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>112</v>
+        <v>42</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3191,6 +3591,31 @@
       <c r="E19" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:22</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>82</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4319
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:00:55</t>
+          <t>Última actualización: 10:38:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 91</t>
+          <t>Total filas: 102</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -883,11 +883,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:33</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>10:41</t>
+          <t>10:38</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2353,16 +2353,16 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:41</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,12 +2373,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>09:14:25</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>90</v>
+        <v>43</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:33</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>10:51</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:33</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>09:14:25</t>
+          <t>10:38:33</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>10:56</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>102</v>
+        <v>17</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:33</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>10:56</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:33</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>11:07</t>
+          <t>11:01</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>09:14:25</t>
+          <t>10:38:33</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>114</v>
+        <v>26</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2553,16 +2553,16 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>11:12</t>
+          <t>11:07</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:33</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>11:23</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2603,16 +2603,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>11:34</t>
+          <t>11:12</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:33</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>95</v>
+        <v>37</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2653,16 +2653,16 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>11:37</t>
+          <t>11:23</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:33</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:24</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>104</v>
+        <v>46</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2703,16 +2703,16 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>11:54</t>
+          <t>11:34</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,23 +2723,298 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
+          <t>10:38:33</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>57</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
           <t>10:00:55</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>95</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>10:38:33</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>11:36</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>58</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>10:38:33</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>11:37</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>59</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>10:38:33</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>66</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>10:38:33</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>76</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>10:38:33</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D96" t="n">
-        <v>115</v>
-      </c>
-      <c r="E96" t="inlineStr">
+      <c r="D102" t="n">
+        <v>77</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>10:38:33</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>86</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>10:38:33</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>97</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>10:38:33</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>106</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>10:38:33</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>116</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>10:38:33</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>118</v>
+      </c>
+      <c r="E107" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2756,7 +3031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2769,14 +3044,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:00:55</t>
+          <t>Última actualización: 10:38:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -2995,7 +3270,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -3020,7 +3295,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -3160,23 +3435,48 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:33</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>57</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10:38:33</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>11:44</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>104</v>
-      </c>
-      <c r="E20" t="inlineStr">
+      <c r="D21" t="n">
+        <v>66</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3193,7 +3493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3206,14 +3506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:00:55</t>
+          <t>Última actualización: 10:38:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3572,7 +3872,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>09:14:25</t>
+          <t>10:38:33</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3586,7 +3886,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>89</v>
+        <v>5</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3614,6 +3914,31 @@
         <v>82</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10:38:33</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>45</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4320
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E107"/>
+  <dimension ref="A1:E116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:38:33</t>
+          <t>Última actualización: 10:56:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 102</t>
+          <t>Total filas: 111</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -883,11 +883,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>11:01</t>
+          <t>10:56</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2528,16 +2528,16 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>11:01</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:33</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>11:07</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:05</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2603,16 +2603,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>11:12</t>
+          <t>11:07</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2653,16 +2653,16 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>11:23</t>
+          <t>11:12</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>11:24</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2703,16 +2703,16 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>11:34</t>
+          <t>11:23</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>11:24</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2753,16 +2753,16 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>11:34</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,12 +2773,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>11:36</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2787,7 +2787,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>11:37</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:36</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2853,16 +2853,16 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>11:54</t>
+          <t>11:37</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>77</v>
+        <v>45</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2903,16 +2903,16 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>97</v>
+        <v>49</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>11:54</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>106</v>
+        <v>58</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>116</v>
+        <v>59</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,23 +2998,248 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
+          <t>10:56:13</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>68</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>10:56:13</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>79</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
           <t>10:38:33</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>106</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>10:56:13</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>89</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>10:56:13</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>12:29</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>93</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>10:56:13</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>98</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>10:56:13</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
         <is>
           <t>12:36</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
+      <c r="C113" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D107" t="n">
-        <v>118</v>
-      </c>
-      <c r="E107" t="inlineStr">
+      <c r="D113" t="n">
+        <v>100</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>10:56:13</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>108</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>10:56:13</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>110</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>10:56:13</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>119</v>
+      </c>
+      <c r="E116" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3031,7 +3256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3044,14 +3269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:38:33</t>
+          <t>Última actualización: 10:56:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3270,7 +3495,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -3295,7 +3520,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -3435,7 +3660,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3449,7 +3674,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3477,6 +3702,56 @@
         <v>66</v>
       </c>
       <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>10:56:13</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>49</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>10:56:13</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>119</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3506,7 +3781,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:38:33</t>
+          <t>Última actualización: 10:56:13</t>
         </is>
       </c>
     </row>
@@ -3922,7 +4197,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3936,7 +4211,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4321
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E116"/>
+  <dimension ref="A1:E119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:56:13</t>
+          <t>Última actualización: 11:13:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 111</t>
+          <t>Total filas: 114</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2812,7 +2812,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2837,7 +2837,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2962,7 +2962,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3012,7 +3012,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,12 +3148,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -3162,7 +3162,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>108</v>
+        <v>81</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3203,16 +3203,16 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,23 +3223,98 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>91</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>11:13:14</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>93</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>11:13:14</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
           <t>12:55</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
+      <c r="C118" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D116" t="n">
-        <v>119</v>
-      </c>
-      <c r="E116" t="inlineStr">
+      <c r="D118" t="n">
+        <v>102</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>11:13:14</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>112</v>
+      </c>
+      <c r="E119" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3269,7 +3344,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:56:13</t>
+          <t>Última actualización: 11:13:14</t>
         </is>
       </c>
     </row>
@@ -3445,7 +3520,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -3470,7 +3545,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -3495,7 +3570,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -3520,7 +3595,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -3660,7 +3735,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3674,7 +3749,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3710,7 +3785,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3724,7 +3799,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3735,7 +3810,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3749,7 +3824,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3781,7 +3856,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:56:13</t>
+          <t>Última actualización: 11:13:14</t>
         </is>
       </c>
     </row>
@@ -4197,7 +4272,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4211,7 +4286,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4322
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E119"/>
+  <dimension ref="A1:E128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:13:14</t>
+          <t>Última actualización: 11:38:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 114</t>
+          <t>Total filas: 123</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2912,7 +2912,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>66</v>
+        <v>6</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2962,7 +2962,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,12 +2998,12 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -3012,7 +3012,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3028,16 +3028,16 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:11</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>106</v>
+        <v>33</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>72</v>
+        <v>37</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>93</v>
+        <v>44</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3153,16 +3153,16 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>100</v>
+        <v>53</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3228,16 +3228,16 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>93</v>
+        <v>56</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,23 +3298,248 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
+          <t>11:38:53</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>12:43</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>65</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
           <t>11:13:14</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr">
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>91</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>11:38:53</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>68</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>11:38:53</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>76</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>11:13:14</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>102</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>11:38:53</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>86</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>11:13:14</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
         <is>
           <t>13:05</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr">
+      <c r="C125" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D119" t="n">
+      <c r="D125" t="n">
         <v>112</v>
       </c>
-      <c r="E119" t="inlineStr">
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>11:38:53</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>97</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>11:38:53</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>105</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>11:38:53</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>113</v>
+      </c>
+      <c r="E128" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3331,7 +3556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3344,14 +3569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:13:14</t>
+          <t>Última actualización: 11:38:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -3520,7 +3745,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -3545,7 +3770,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -3760,7 +3985,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10:38:33</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3774,7 +3999,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>66</v>
+        <v>6</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3810,23 +4035,73 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>11:38:53</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>76</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>11:13:14</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>12:55</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D24" t="n">
         <v>102</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>11:38:53</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>113</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3843,7 +4118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3856,14 +4131,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:13:14</t>
+          <t>Última actualización: 11:38:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -4289,6 +4564,31 @@
         <v>10</v>
       </c>
       <c r="E21" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>11:38:53</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>104</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4323
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E128"/>
+  <dimension ref="A1:E133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:38:53</t>
+          <t>Última actualización: 11:55:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 123</t>
+          <t>Total filas: 128</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -883,11 +883,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>12:03</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,12 +3023,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>12:11</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:11</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3128,16 +3128,16 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>93</v>
+        <v>29</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,12 +3273,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>12:43</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3353,16 +3353,16 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:46</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>86</v>
+        <v>59</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3453,16 +3453,16 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,23 +3523,148 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
+          <t>11:55:42</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>80</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>11:55:42</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>87</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
           <t>11:38:53</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr">
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>105</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>11:55:42</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>89</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>11:55:42</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
         <is>
           <t>13:31</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr">
+      <c r="C132" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D128" t="n">
-        <v>113</v>
-      </c>
-      <c r="E128" t="inlineStr">
+      <c r="D132" t="n">
+        <v>96</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>11:55:42</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>109</v>
+      </c>
+      <c r="E133" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3569,7 +3694,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:38:53</t>
+          <t>Última actualización: 11:55:42</t>
         </is>
       </c>
     </row>
@@ -4035,7 +4160,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4049,7 +4174,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4085,7 +4210,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4099,7 +4224,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4118,7 +4243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4131,14 +4256,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:38:53</t>
+          <t>Última actualización: 11:55:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -4572,7 +4697,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4586,11 +4711,36 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>11:55:42</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>114</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4324
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E133"/>
+  <dimension ref="A1:E142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:55:42</t>
+          <t>Última actualización: 12:10:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 128</t>
+          <t>Total filas: 137</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -883,11 +883,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3073,12 +3073,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>12:11</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3103,16 +3103,16 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:11</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,12 +3148,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -3162,7 +3162,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>93</v>
+        <v>29</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3303,16 +3303,16 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>100</v>
+        <v>22</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>12:43</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>51</v>
+        <v>100</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>102</v>
+        <v>34</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:46</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>69</v>
+        <v>36</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>112</v>
+        <v>59</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3553,16 +3553,16 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>105</v>
+        <v>55</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3628,16 +3628,16 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:22</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,23 +3648,248 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
+          <t>11:38:53</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>105</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>12:10:01</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>74</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>12:10:01</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>74</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
           <t>11:55:42</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr">
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>96</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>12:10:01</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>82</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>11:55:42</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
         <is>
           <t>13:44</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr">
+      <c r="C138" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D133" t="n">
+      <c r="D138" t="n">
         <v>109</v>
       </c>
-      <c r="E133" t="inlineStr">
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>12:10:01</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>95</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>12:10:01</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>105</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>12:10:01</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>14:01</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>111</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>12:10:01</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>114</v>
+      </c>
+      <c r="E142" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3681,7 +3906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3694,14 +3919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:55:42</t>
+          <t>Última actualización: 12:10:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -4185,7 +4410,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4199,7 +4424,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>102</v>
+        <v>45</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4227,6 +4452,31 @@
         <v>96</v>
       </c>
       <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>12:10:01</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>82</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4243,7 +4493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4256,14 +4506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:55:42</t>
+          <t>Última actualización: 12:10:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -4722,23 +4972,73 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>12:10:01</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>73</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>11:55:42</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>13:49</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D24" t="n">
         <v>114</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>12:10:01</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>100</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4325
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E142"/>
+  <dimension ref="A1:E151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:10:01</t>
+          <t>Última actualización: 12:33:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 137</t>
+          <t>Total filas: 146</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>10:56:13</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>10:56:13</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>12:43</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,12 +3448,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -3462,7 +3462,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:46</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,12 +3523,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>69</v>
+        <v>22</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,12 +3573,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>87</v>
+        <v>42</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>105</v>
+        <v>48</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,12 +3673,12 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:22</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -3687,7 +3687,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,12 +3698,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:38:53</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -3712,7 +3712,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>74</v>
+        <v>105</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3753,16 +3753,16 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3803,16 +3803,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:44</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>14:01</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>111</v>
+        <v>72</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,23 +3873,248 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
+          <t>12:33:16</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>82</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>12:33:16</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>83</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
           <t>12:10:01</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr">
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>14:01</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>111</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>12:33:16</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
         <is>
           <t>14:04</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr">
+      <c r="C145" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D142" t="n">
-        <v>114</v>
-      </c>
-      <c r="E142" t="inlineStr">
+      <c r="D145" t="n">
+        <v>91</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>12:33:16</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>98</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>12:33:16</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>101</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>12:33:16</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>101</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>12:33:16</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>101</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>12:33:16</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>112</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>12:33:16</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>118</v>
+      </c>
+      <c r="E151" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3919,7 +4144,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:10:01</t>
+          <t>Última actualización: 12:33:16</t>
         </is>
       </c>
     </row>
@@ -4410,7 +4635,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4424,7 +4649,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4435,7 +4660,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4449,7 +4674,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>96</v>
+        <v>58</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4506,7 +4731,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:10:01</t>
+          <t>Última actualización: 12:33:16</t>
         </is>
       </c>
     </row>
@@ -4972,7 +5197,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4986,7 +5211,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -5022,7 +5247,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5036,7 +5261,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4326
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E151"/>
+  <dimension ref="A1:E157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:33:16</t>
+          <t>Última actualización: 12:51:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 146</t>
+          <t>Total filas: 152</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>69</v>
+        <v>13</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3637,7 +3637,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3662,7 +3662,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>11:38:53</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3712,7 +3712,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>105</v>
+        <v>32</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3823,7 +3823,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3837,7 +3837,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>109</v>
+        <v>53</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3948,12 +3948,12 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -3962,7 +3962,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3978,16 +3978,16 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>112</v>
+        <v>83</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,23 +4098,173 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
+          <t>12:51:54</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>83</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>12:51:54</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>85</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>12:51:54</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>93</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
           <t>12:33:16</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>112</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>12:51:54</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
         <is>
           <t>14:31</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
+      <c r="C155" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D151" t="n">
-        <v>118</v>
-      </c>
-      <c r="E151" t="inlineStr">
+      <c r="D155" t="n">
+        <v>100</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>12:51:54</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>103</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>12:51:54</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>112</v>
+      </c>
+      <c r="E157" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4131,7 +4281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4144,14 +4294,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:33:16</t>
+          <t>Última actualización: 12:51:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -4610,7 +4760,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4624,7 +4774,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4660,7 +4810,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4674,7 +4824,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4702,6 +4852,31 @@
         <v>82</v>
       </c>
       <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>12:51:54</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>103</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4718,7 +4893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4731,14 +4906,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:33:16</t>
+          <t>Última actualización: 12:51:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -5172,12 +5347,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -5186,7 +5361,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>87</v>
+        <v>3</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -5197,12 +5372,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>11:55:42</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:22</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -5211,7 +5386,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>50</v>
+        <v>87</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -5222,50 +5397,100 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>13:49</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>114</v>
+        <v>50</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>12:51:54</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>58</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>12:33:16</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>13:50</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D26" t="n">
         <v>77</v>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>12:51:54</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>111</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4327
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E157"/>
+  <dimension ref="A1:E162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:51:54</t>
+          <t>Última actualización: 13:10:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 152</t>
+          <t>Total filas: 157</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3637,7 +3637,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3662,7 +3662,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3823,7 +3823,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3837,7 +3837,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>91</v>
+        <v>54</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:10</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4028,16 +4028,16 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,12 +4048,12 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -4062,7 +4062,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4087,7 +4087,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>93</v>
+        <v>66</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,12 +4173,12 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>112</v>
+        <v>74</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>103</v>
+        <v>81</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,23 +4248,148 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
+          <t>13:10:37</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>84</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
           <t>12:51:54</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr">
+      <c r="B158" t="inlineStr">
         <is>
           <t>14:43</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr">
+      <c r="C158" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D157" t="n">
+      <c r="D158" t="n">
         <v>112</v>
       </c>
-      <c r="E157" t="inlineStr">
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>13:10:37</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>94</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>13:10:37</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>104</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>13:10:37</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>111</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>13:10:37</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>114</v>
+      </c>
+      <c r="E162" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4281,7 +4406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4294,14 +4419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:51:54</t>
+          <t>Última actualización: 13:10:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -4810,7 +4935,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4824,7 +4949,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4860,7 +4985,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4874,9 +4999,59 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:10:37</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>104</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13:10:37</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>114</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4906,7 +5081,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:51:54</t>
+          <t>Última actualización: 13:10:37</t>
         </is>
       </c>
     </row>
@@ -5372,7 +5547,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11:55:42</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5386,7 +5561,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>87</v>
+        <v>12</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -5447,7 +5622,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5461,7 +5636,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>77</v>
+        <v>40</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -5472,7 +5647,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5486,7 +5661,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4328
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E162"/>
+  <dimension ref="A1:E171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:10:37</t>
+          <t>Última actualización: 13:42:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 157</t>
+          <t>Total filas: 166</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>22</v>
+        <v>95</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3823,7 +3823,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3837,7 +3837,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,12 +3923,12 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>14:01</t>
+          <t>13:59</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -3937,7 +3937,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>111</v>
+        <v>17</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>72</v>
+        <v>111</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,12 +3973,12 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:10</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>81</v>
+        <v>29</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4178,16 +4178,16 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>112</v>
+        <v>35</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4228,16 +4228,16 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>84</v>
+        <v>43</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>112</v>
+        <v>49</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4303,16 +4303,16 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>104</v>
+        <v>53</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,23 +4373,248 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
+          <t>13:42:16</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>62</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
           <t>13:10:37</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr">
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>104</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>13:42:16</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>73</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>13:42:16</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>78</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>13:10:37</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>111</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>13:10:37</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
         <is>
           <t>15:04</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr">
+      <c r="C167" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D162" t="n">
+      <c r="D167" t="n">
         <v>114</v>
       </c>
-      <c r="E162" t="inlineStr">
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>13:42:16</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>83</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>13:42:16</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>93</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>13:42:16</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>102</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>13:42:16</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>113</v>
+      </c>
+      <c r="E171" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4406,7 +4631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4419,14 +4644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:10:37</t>
+          <t>Última actualización: 13:42:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -5010,21 +5235,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>104</v>
+        <v>53</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5040,18 +5265,118 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>104</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>13:42:16</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>73</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>13:10:37</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>15:04</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D31" t="n">
         <v>114</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>13:42:16</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>83</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>13:42:16</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>113</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5068,7 +5393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5081,14 +5406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:10:37</t>
+          <t>Última actualización: 13:42:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -5622,7 +5947,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5636,7 +5961,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -5666,6 +5991,56 @@
       <c r="E27" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:42:16</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>61</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13:42:16</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>101</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4329
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E171"/>
+  <dimension ref="A1:E177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:42:16</t>
+          <t>Última actualización: 14:00:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 166</t>
+          <t>Total filas: 172</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3962,7 +3962,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>111</v>
+        <v>1</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,12 +3973,12 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>72</v>
+        <v>2</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,12 +3998,12 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -4012,7 +4012,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>22</v>
+        <v>72</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:10</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>81</v>
+        <v>11</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,12 +4098,12 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -4112,7 +4112,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4162,7 +4162,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,12 +4173,12 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>66</v>
+        <v>101</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,12 +4198,12 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -4212,7 +4212,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>74</v>
+        <v>17</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,12 +4248,12 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -4262,7 +4262,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>43</v>
+        <v>74</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>84</v>
+        <v>31</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,12 +4323,12 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>112</v>
+        <v>35</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,12 +4373,12 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -4387,7 +4387,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>62</v>
+        <v>112</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>104</v>
+        <v>44</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,12 +4423,12 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>73</v>
+        <v>104</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,12 +4473,12 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -4487,7 +4487,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>111</v>
+        <v>56</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>114</v>
+        <v>78</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>83</v>
+        <v>111</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>102</v>
+        <v>65</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,23 +4598,173 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>66</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>14:00:16</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>75</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>14:00:16</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>84</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>14:00:16</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
           <t>15:35</t>
         </is>
       </c>
-      <c r="C171" t="inlineStr">
+      <c r="C174" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D171" t="n">
-        <v>113</v>
-      </c>
-      <c r="E171" t="inlineStr">
+      <c r="D174" t="n">
+        <v>95</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>14:00:16</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>105</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>14:00:16</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>115</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>14:00:16</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>116</v>
+      </c>
+      <c r="E177" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4644,7 +4794,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:42:16</t>
+          <t>Última actualización: 14:00:16</t>
         </is>
       </c>
     </row>
@@ -5235,7 +5385,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5249,7 +5399,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5285,7 +5435,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5299,7 +5449,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5335,7 +5485,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5349,7 +5499,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5360,7 +5510,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5374,7 +5524,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5406,7 +5556,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:42:16</t>
+          <t>Última actualización: 14:00:16</t>
         </is>
       </c>
     </row>
@@ -5997,7 +6147,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -6011,7 +6161,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -6022,7 +6172,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -6036,7 +6186,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4330
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E177"/>
+  <dimension ref="A1:E184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:00:16</t>
+          <t>Última actualización: 14:19:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 172</t>
+          <t>Total filas: 179</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>22</v>
+        <v>95</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4183,11 +4183,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,12 +4273,12 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4303,16 +4303,16 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>84</v>
+        <v>31</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,12 +4348,12 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -4362,7 +4362,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>112</v>
+        <v>35</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,12 +4398,12 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>44</v>
+        <v>112</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>104</v>
+        <v>25</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,12 +4448,12 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -4462,7 +4462,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4478,16 +4478,16 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,12 +4498,12 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -4512,7 +4512,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>78</v>
+        <v>56</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,12 +4523,12 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>114</v>
+        <v>42</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,12 +4573,12 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4603,16 +4603,16 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4728,16 +4728,16 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,23 +4748,198 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
+          <t>14:19:40</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>82</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>14:19:40</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>85</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
           <t>14:00:16</t>
         </is>
       </c>
-      <c r="B177" t="inlineStr">
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>105</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>14:19:40</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>89</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>14:19:40</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>96</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>14:00:16</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
         <is>
           <t>15:56</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
+      <c r="C182" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D177" t="n">
+      <c r="D182" t="n">
         <v>116</v>
       </c>
-      <c r="E177" t="inlineStr">
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>14:19:40</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>105</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>14:19:40</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>115</v>
+      </c>
+      <c r="E184" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4781,7 +4956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4794,14 +4969,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:00:16</t>
+          <t>Última actualización: 14:19:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5535,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5374,7 +5549,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -5410,7 +5585,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5424,7 +5599,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>104</v>
+        <v>35</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5460,7 +5635,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5474,7 +5649,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>114</v>
+        <v>45</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -5510,23 +5685,48 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>14:19:40</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>75</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>14:00:16</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>15:35</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D34" t="n">
         <v>95</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5543,7 +5743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5556,14 +5756,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:00:16</t>
+          <t>Última actualización: 14:19:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6322,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -6136,7 +6336,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>92</v>
+        <v>23</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -6172,25 +6372,75 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>14:19:40</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>63</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>14:00:16</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>15:23</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D30" t="n">
         <v>83</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>14:19:40</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>16:02</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>103</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4331
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E184"/>
+  <dimension ref="A1:E190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:19:40</t>
+          <t>Última actualización: 14:37:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 179</t>
+          <t>Total filas: 185</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4183,11 +4183,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>12:51:54</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>112</v>
+        <v>1</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,12 +4423,12 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>12:51:54</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>25</v>
+        <v>112</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,12 +4473,12 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -4487,7 +4487,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>56</v>
+        <v>18</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,12 +4523,12 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>13:42:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>78</v>
+        <v>56</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,12 +4548,12 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>13:42:16</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -4562,7 +4562,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,12 +4598,12 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -4612,7 +4612,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>65</v>
+        <v>27</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,12 +4723,12 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -4737,7 +4737,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>82</v>
+        <v>58</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,12 +4798,12 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -4812,7 +4812,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>105</v>
+        <v>67</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4853,16 +4853,16 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:52</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>116</v>
+        <v>75</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>105</v>
+        <v>78</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,23 +4923,173 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>116</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>14:37:21</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>15:58</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>81</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>14:37:21</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>87</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>14:37:21</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
           <t>16:14</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr">
+      <c r="C187" t="inlineStr">
         <is>
           <t>17X38_ROMERO</t>
         </is>
       </c>
-      <c r="D184" t="n">
-        <v>115</v>
-      </c>
-      <c r="E184" t="inlineStr">
+      <c r="D187" t="n">
+        <v>97</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>14:37:21</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>107</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>14:37:21</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>117</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>14:37:21</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>118</v>
+      </c>
+      <c r="E190" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4969,7 +5119,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:19:40</t>
+          <t>Última actualización: 14:37:21</t>
         </is>
       </c>
     </row>
@@ -5610,7 +5760,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5624,7 +5774,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>55</v>
+        <v>18</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5635,7 +5785,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5649,7 +5799,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -5710,7 +5860,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5724,7 +5874,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>95</v>
+        <v>58</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -5743,7 +5893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5756,14 +5906,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:19:40</t>
+          <t>Última actualización: 14:37:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -6322,12 +6472,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>14:42</t>
+          <t>14:39</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -6336,7 +6486,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -6347,12 +6497,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:42</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -6361,7 +6511,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -6372,37 +6522,37 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -6411,7 +6561,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -6422,25 +6572,100 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>14:37:21</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>46</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>14:19:40</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>16:02</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D32" t="n">
         <v>103</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>14:37:21</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>86</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>14:37:21</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>113</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4332
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E190"/>
+  <dimension ref="A1:E193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:37:21</t>
+          <t>Última actualización: 14:51:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 185</t>
+          <t>Total filas: 188</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>22</v>
+        <v>95</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4512,7 +4512,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4612,7 +4612,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4712,7 +4712,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4748,7 +4748,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -4762,7 +4762,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4787,7 +4787,7 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4812,7 +4812,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4873,12 +4873,12 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>15:52</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4903,16 +4903,16 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:52</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>116</v>
+        <v>64</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>81</v>
+        <v>116</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5003,16 +5003,16 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>15:58</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>107</v>
+        <v>73</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>117</v>
+        <v>83</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,23 +5073,98 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>93</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>14:51:24</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>103</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>14:51:24</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
           <t>16:35</t>
         </is>
       </c>
-      <c r="C190" t="inlineStr">
+      <c r="C192" t="inlineStr">
         <is>
           <t>83_ALUAR</t>
         </is>
       </c>
-      <c r="D190" t="n">
-        <v>118</v>
-      </c>
-      <c r="E190" t="inlineStr">
+      <c r="D192" t="n">
+        <v>104</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>14:51:24</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>113</v>
+      </c>
+      <c r="E193" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5119,7 +5194,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:37:21</t>
+          <t>Última actualización: 14:51:24</t>
         </is>
       </c>
     </row>
@@ -5760,7 +5835,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5774,7 +5849,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5785,7 +5860,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5799,7 +5874,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -5860,7 +5935,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5874,7 +5949,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -5906,7 +5981,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:37:21</t>
+          <t>Última actualización: 14:51:24</t>
         </is>
       </c>
     </row>
@@ -6572,7 +6647,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -6586,7 +6661,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -6622,7 +6697,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6636,7 +6711,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6647,7 +6722,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6661,7 +6736,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4333
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E193"/>
+  <dimension ref="A1:E199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:51:24</t>
+          <t>Última actualización: 15:11:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 188</t>
+          <t>Total filas: 194</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>22</v>
+        <v>95</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4183,11 +4183,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>75</v>
+        <v>13</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,12 +4748,12 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -4762,7 +4762,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,12 +4823,12 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -4837,7 +4837,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>105</v>
+        <v>53</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,12 +4873,12 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>15:50</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,12 +4898,12 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>15:52</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -4912,7 +4912,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:52</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>116</v>
+        <v>75</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>81</v>
+        <v>116</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>73</v>
+        <v>46</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>15:58</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>93</v>
+        <v>53</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>103</v>
+        <v>63</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:16</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>104</v>
+        <v>65</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,23 +5148,173 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>73</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>15:11:16</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>83</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>15:11:16</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>84</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>15:11:16</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>90</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>15:11:16</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
           <t>16:44</t>
         </is>
       </c>
-      <c r="C193" t="inlineStr">
+      <c r="C197" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D193" t="n">
-        <v>113</v>
-      </c>
-      <c r="E193" t="inlineStr">
+      <c r="D197" t="n">
+        <v>93</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>15:11:16</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>104</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>15:11:16</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>108</v>
+      </c>
+      <c r="E199" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5181,7 +5331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5194,14 +5344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:51:24</t>
+          <t>Última actualización: 15:11:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -5910,21 +6060,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>75</v>
+        <v>2</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5935,23 +6085,48 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>75</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>15:11:16</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>15:35</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>44</v>
-      </c>
-      <c r="E34" t="inlineStr">
+      <c r="D35" t="n">
+        <v>24</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5968,7 +6143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5981,14 +6156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:51:24</t>
+          <t>Última actualización: 15:11:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -6647,7 +6822,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -6661,7 +6836,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -6697,7 +6872,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6711,7 +6886,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6739,6 +6914,31 @@
         <v>99</v>
       </c>
       <c r="E34" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>15:11:16</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>83</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4334
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E199"/>
+  <dimension ref="A1:E208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:11:16</t>
+          <t>Última actualización: 15:47:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 194</t>
+          <t>Total filas: 203</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -883,11 +883,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4183,11 +4183,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>14:19:40</t>
+          <t>15:47:06</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>89</v>
+        <v>0</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,12 +4898,12 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>14:19:40</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>15:50</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -4912,7 +4912,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,12 +4923,12 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>14:51:24</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -4937,7 +4937,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,12 +4948,12 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>15:52</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -4962,7 +4962,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>15:47:06</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:52</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>15:47:06</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>116</v>
+        <v>8</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>46</v>
+        <v>116</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,12 +5048,12 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>14:37:21</t>
+          <t>15:47:06</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -5062,7 +5062,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>81</v>
+        <v>10</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>14:37:21</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:58</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>15:47:06</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>63</v>
+        <v>17</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>15:47:06</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>16:16</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>65</v>
+        <v>27</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>15:47:06</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:16</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>73</v>
+        <v>29</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5178,16 +5178,16 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,21 +5198,21 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>15:47:06</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>15:47:06</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>90</v>
+        <v>47</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>15:47:06</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>93</v>
+        <v>48</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5278,16 +5278,16 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,23 +5298,248 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
+          <t>15:47:06</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>57</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>15:47:06</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>68</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
           <t>15:11:16</t>
         </is>
       </c>
-      <c r="B199" t="inlineStr">
+      <c r="B201" t="inlineStr">
         <is>
           <t>16:59</t>
         </is>
       </c>
-      <c r="C199" t="inlineStr">
+      <c r="C201" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D199" t="n">
+      <c r="D201" t="n">
         <v>108</v>
       </c>
-      <c r="E199" t="inlineStr">
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>15:47:06</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>78</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>15:47:06</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>88</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>15:47:06</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>97</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>15:47:06</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>105</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>15:47:06</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>108</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>15:47:06</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>110</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>15:47:06</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>118</v>
+      </c>
+      <c r="E208" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5331,7 +5556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5344,14 +5569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:11:16</t>
+          <t>Última actualización: 15:47:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -6127,6 +6352,56 @@
         <v>24</v>
       </c>
       <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>15:47:06</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>88</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>15:47:06</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>118</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6143,7 +6418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6156,14 +6431,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:11:16</t>
+          <t>Última actualización: 15:47:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -6872,7 +7147,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>15:47:06</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6886,7 +7161,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6897,7 +7172,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>14:51:24</t>
+          <t>15:47:06</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6911,7 +7186,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>99</v>
+        <v>43</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -6941,6 +7216,31 @@
       <c r="E35" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>15:47:06</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>96</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4335
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E208"/>
+  <dimension ref="A1:E212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:47:06</t>
+          <t>Última actualización: 16:04:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 203</t>
+          <t>Total filas: 207</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -883,11 +883,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5112,7 +5112,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>16:16</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:16</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>73</v>
+        <v>12</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,12 +5198,12 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>90</v>
+        <v>31</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>108</v>
+        <v>51</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,12 +5373,12 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -5387,7 +5387,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>78</v>
+        <v>108</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>88</v>
+        <v>61</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>97</v>
+        <v>71</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,21 +5498,21 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>110</v>
+        <v>91</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5528,18 +5528,118 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>110</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>16:04:08</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>17:41</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>97</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>16:04:08</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
           <t>17:45</t>
         </is>
       </c>
-      <c r="C208" t="inlineStr">
+      <c r="C210" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D208" t="n">
-        <v>118</v>
-      </c>
-      <c r="E208" t="inlineStr">
+      <c r="D210" t="n">
+        <v>101</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>16:04:08</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>111</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>16:04:08</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>116</v>
+      </c>
+      <c r="E212" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5556,7 +5656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5569,14 +5669,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:47:06</t>
+          <t>Última actualización: 16:04:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -5745,7 +5845,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -5770,7 +5870,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -5795,7 +5895,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -5820,7 +5920,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -6360,7 +6460,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6374,7 +6474,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6385,7 +6485,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6399,9 +6499,34 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>118</v>
+        <v>101</v>
       </c>
       <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>16:04:08</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>111</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6418,7 +6543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6431,14 +6556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:47:06</t>
+          <t>Última actualización: 16:04:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -7172,37 +7297,37 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-40 Y 115</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -7211,7 +7336,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>83</v>
+        <v>26</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -7222,23 +7347,48 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>83</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>16:04:08</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>17:23</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>96</v>
-      </c>
-      <c r="E36" t="inlineStr">
+      <c r="D37" t="n">
+        <v>79</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4336
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E212"/>
+  <dimension ref="A1:E223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:04:08</t>
+          <t>Última actualización: 16:27:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 207</t>
+          <t>Total filas: 218</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5287,7 +5287,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,7 +5298,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5312,7 +5312,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5337,7 +5337,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>108</v>
+        <v>28</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,12 +5398,12 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -5412,7 +5412,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>61</v>
+        <v>108</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>71</v>
+        <v>37</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5453,16 +5453,16 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>88</v>
+        <v>47</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5503,16 +5503,16 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>91</v>
+        <v>71</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>110</v>
+        <v>57</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5578,16 +5578,16 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>111</v>
+        <v>68</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,23 +5623,298 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
+          <t>16:27:50</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>68</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>15:47:06</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>110</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>16:27:50</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>17:39</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>72</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
           <t>16:04:08</t>
         </is>
       </c>
-      <c r="B212" t="inlineStr">
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>17:41</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>97</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>16:27:50</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>77</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>16:04:08</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>101</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>16:27:50</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>87</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>16:04:08</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>111</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>16:04:08</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
         <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="C212" t="inlineStr">
+      <c r="C220" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D212" t="n">
+      <c r="D220" t="n">
         <v>116</v>
       </c>
-      <c r="E212" t="inlineStr">
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>16:27:50</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>18:03</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>96</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>16:27:50</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>107</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>16:27:50</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>117</v>
+      </c>
+      <c r="E223" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5656,7 +5931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5669,14 +5944,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:04:08</t>
+          <t>Última actualización: 16:27:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -5895,7 +6170,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -5920,7 +6195,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -6460,12 +6735,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -6474,7 +6749,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6490,16 +6765,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>101</v>
+        <v>71</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6510,23 +6785,123 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>16:27:50</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>77</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>16:04:08</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>101</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>16:27:50</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>87</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>16:04:08</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
         <is>
           <t>17:55</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D41" t="n">
         <v>111</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>16:27:50</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>107</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6543,7 +6918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6556,14 +6931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:04:08</t>
+          <t>Última actualización: 16:27:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -7322,12 +7697,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:29</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -7336,7 +7711,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -7347,12 +7722,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -7361,7 +7736,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>83</v>
+        <v>26</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -7372,23 +7747,73 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>15:11:16</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>83</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>16:27:50</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>55</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>16:04:08</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>17:23</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D37" t="n">
+      <c r="D39" t="n">
         <v>79</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4337
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E223"/>
+  <dimension ref="A1:E230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:27:51</t>
+          <t>Última actualización: 16:42:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 218</t>
+          <t>Total filas: 225</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4183,11 +4183,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:43</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>108</v>
+        <v>13</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,12 +5423,12 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>37</v>
+        <v>108</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,12 +5448,12 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -5462,7 +5462,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,12 +5498,12 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>17:26</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>68</v>
+        <v>88</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,12 +5623,12 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -5637,7 +5637,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>15:47:06</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>110</v>
+        <v>53</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5678,16 +5678,16 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>17:39</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,12 +5698,12 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -5712,7 +5712,7 @@
         </is>
       </c>
       <c r="D215" t="n">
-        <v>97</v>
+        <v>55</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5728,16 +5728,16 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:39</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5753,16 +5753,16 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5778,16 +5778,16 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>17:54</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>111</v>
+        <v>63</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:54</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>18:03</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>18:14</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5903,18 +5903,193 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
+          <t>18:03</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>96</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>16:42:10</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>82</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>16:27:50</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>107</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>16:42:10</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>93</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>16:27:50</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
           <t>18:24</t>
         </is>
       </c>
-      <c r="C223" t="inlineStr">
+      <c r="C227" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D223" t="n">
+      <c r="D227" t="n">
         <v>117</v>
       </c>
-      <c r="E223" t="inlineStr">
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>16:42:10</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>103</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>16:42:10</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>112</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>16:42:10</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>114</v>
+      </c>
+      <c r="E230" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5931,7 +6106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5944,14 +6119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:27:51</t>
+          <t>Última actualización: 16:42:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -6760,7 +6935,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6774,7 +6949,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6810,7 +6985,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6824,7 +6999,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>101</v>
+        <v>63</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6860,7 +7035,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -6874,7 +7049,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>111</v>
+        <v>73</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -6902,6 +7077,31 @@
         <v>107</v>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>16:42:10</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>93</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6931,7 +7131,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:27:51</t>
+          <t>Última actualización: 16:42:10</t>
         </is>
       </c>
     </row>
@@ -7797,7 +7997,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7811,7 +8011,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4338
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E230"/>
+  <dimension ref="A1:E234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:42:10</t>
+          <t>Última actualización: 16:55:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 225</t>
+          <t>Total filas: 229</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5412,7 +5412,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>15:11:16</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,12 +5448,12 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>15:11:16</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -5462,7 +5462,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>37</v>
+        <v>108</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,12 +5473,12 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,21 +5498,21 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,12 +5523,12 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -5537,7 +5537,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>17:26</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,12 +5623,12 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -5637,7 +5637,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>53</v>
+        <v>88</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,12 +5673,12 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:42:10</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -5687,7 +5687,7 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>17:39</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,12 +5748,12 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -5762,7 +5762,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5778,16 +5778,16 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:39</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>63</v>
+        <v>97</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>17:54</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>87</v>
+        <v>49</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5853,16 +5853,16 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:54</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>18:03</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>96</v>
+        <v>60</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,12 +5923,12 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -5937,7 +5937,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5953,16 +5953,16 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>18:14</t>
+          <t>18:03</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -6003,16 +6003,16 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>112</v>
+        <v>87</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,23 +6073,123 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
+          <t>16:55:20</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>89</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
           <t>16:42:10</t>
         </is>
       </c>
-      <c r="B230" t="inlineStr">
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>103</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>16:55:20</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>99</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>16:55:20</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
         <is>
           <t>18:36</t>
         </is>
       </c>
-      <c r="C230" t="inlineStr">
+      <c r="C233" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D230" t="n">
-        <v>114</v>
-      </c>
-      <c r="E230" t="inlineStr">
+      <c r="D233" t="n">
+        <v>101</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>16:55:20</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>109</v>
+      </c>
+      <c r="E234" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6119,7 +6219,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:42:10</t>
+          <t>Última actualización: 16:55:20</t>
         </is>
       </c>
     </row>
@@ -6935,7 +7035,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6949,7 +7049,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6960,7 +7060,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6974,7 +7074,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>77</v>
+        <v>49</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -7035,7 +7135,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7049,7 +7149,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -7085,7 +7185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7099,7 +7199,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -7118,7 +7218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7131,14 +7231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:42:10</t>
+          <t>Última actualización: 16:55:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -7997,7 +8097,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -8011,9 +8111,34 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>16:55:20</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>110</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4339
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E234"/>
+  <dimension ref="A1:E238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:55:20</t>
+          <t>Última actualización: 17:08:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 229</t>
+          <t>Total filas: 233</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5562,7 +5562,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,7 +5598,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -5612,7 +5612,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>59</v>
+        <v>18</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5637,7 +5637,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>68</v>
+        <v>27</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>40</v>
+        <v>68</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5762,7 +5762,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5848,7 +5848,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6037,7 +6037,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6112,7 +6112,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>103</v>
+        <v>77</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:26</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,23 +6173,123 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>88</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>17:08:17</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
           <t>18:44</t>
         </is>
       </c>
-      <c r="C234" t="inlineStr">
+      <c r="C235" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D234" t="n">
-        <v>109</v>
-      </c>
-      <c r="E234" t="inlineStr">
+      <c r="D235" t="n">
+        <v>96</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>17:08:17</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>106</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>17:08:17</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>112</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>17:08:17</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>117</v>
+      </c>
+      <c r="E238" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6206,7 +6306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6219,14 +6319,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:55:20</t>
+          <t>Última actualización: 17:08:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7135,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7049,7 +7149,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -7085,7 +7185,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:42:10</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7099,7 +7199,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -7135,7 +7235,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7149,7 +7249,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -7185,7 +7285,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7199,9 +7299,34 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>17:08:17</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>112</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7231,7 +7356,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:55:20</t>
+          <t>Última actualización: 17:08:17</t>
         </is>
       </c>
     </row>
@@ -8097,7 +8222,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -8111,7 +8236,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -8122,7 +8247,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -8136,7 +8261,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4340
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E238"/>
+  <dimension ref="A1:E248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:08:17</t>
+          <t>Última actualización: 17:33:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 233</t>
+          <t>Total filas: 243</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>22</v>
+        <v>95</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4183,11 +4183,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5712,7 +5712,7 @@
         </is>
       </c>
       <c r="D215" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5748,12 +5748,12 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -5762,7 +5762,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,12 +5773,12 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>17:39</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -5787,7 +5787,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,12 +5798,12 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:39</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -5812,7 +5812,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>97</v>
+        <v>72</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>49</v>
+        <v>97</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,12 +5848,12 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>17:54</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>87</v>
+        <v>37</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,12 +5898,12 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:54</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>16:04:08</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>116</v>
+        <v>47</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,12 +5948,12 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>16:04:08</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>18:03</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,12 +5973,12 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>18:03</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>18:14</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>107</v>
+        <v>56</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,12 +6023,12 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -6037,7 +6037,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:08:17</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>89</v>
+        <v>48</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>16:55:20</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>18:26</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6153,16 +6153,16 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6178,16 +6178,16 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:26</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>96</v>
+        <v>61</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>106</v>
+        <v>63</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:43</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>112</v>
+        <v>70</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6278,18 +6278,268 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>96</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>17:33:57</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>81</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>17:33:57</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>86</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>17:08:17</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>112</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>17:33:57</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>91</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>17:08:17</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
           <t>19:05</t>
         </is>
       </c>
-      <c r="C238" t="inlineStr">
+      <c r="C243" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D238" t="n">
+      <c r="D243" t="n">
         <v>117</v>
       </c>
-      <c r="E238" t="inlineStr">
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>17:33:57</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>19:11</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>98</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>17:33:57</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>103</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>17:33:57</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>103</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>17:33:57</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>110</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>17:33:57</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>111</v>
+      </c>
+      <c r="E248" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6306,7 +6556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6319,14 +6569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:08:17</t>
+          <t>Última actualización: 17:33:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -7160,7 +7410,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16:55:20</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7174,7 +7424,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -7210,7 +7460,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7224,7 +7474,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>87</v>
+        <v>21</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -7260,7 +7510,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7274,7 +7524,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>107</v>
+        <v>41</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -7310,23 +7560,73 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>17:33:57</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>86</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>17:08:17</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D44" t="n">
+      <c r="D45" t="n">
         <v>112</v>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>17:33:57</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>111</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7343,7 +7643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7356,14 +7656,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:08:17</t>
+          <t>Última actualización: 17:33:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -8247,25 +8547,75 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>17:33:57</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>71</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>17:08:17</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>18:45</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D40" t="n">
+      <c r="D41" t="n">
         <v>97</v>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>17:33:57</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>19:14</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>101</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4341
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E248"/>
+  <dimension ref="A1:E253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:33:57</t>
+          <t>Última actualización: 17:52:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 243</t>
+          <t>Total filas: 248</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4183,11 +4183,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5937,7 +5937,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>47</v>
+        <v>3</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6012,7 +6012,7 @@
         </is>
       </c>
       <c r="D227" t="n">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6048,7 +6048,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -6062,7 +6062,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,7 +6073,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -6087,7 +6087,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6137,7 +6137,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6212,7 +6212,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -6237,7 +6237,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6273,7 +6273,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -6287,7 +6287,7 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>96</v>
+        <v>52</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -6312,7 +6312,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6348,7 +6348,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -6362,7 +6362,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>112</v>
+        <v>68</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,7 +6373,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -6387,7 +6387,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:13</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>103</v>
+        <v>81</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -6487,7 +6487,7 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,21 +6498,21 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>110</v>
+        <v>84</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6528,18 +6528,143 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>110</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>17:33:57</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
           <t>19:24</t>
         </is>
       </c>
-      <c r="C248" t="inlineStr">
+      <c r="C249" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D248" t="n">
+      <c r="D249" t="n">
         <v>111</v>
       </c>
-      <c r="E248" t="inlineStr">
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>17:52:25</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>92</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>17:52:25</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>93</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>17:52:25</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>117</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>17:52:25</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>118</v>
+      </c>
+      <c r="E253" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6556,7 +6681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6569,14 +6694,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:33:57</t>
+          <t>Última actualización: 17:52:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -7485,7 +7610,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7499,7 +7624,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>47</v>
+        <v>3</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -7535,7 +7660,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7549,7 +7674,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -7585,7 +7710,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7599,7 +7724,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>112</v>
+        <v>68</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -7627,6 +7752,31 @@
         <v>111</v>
       </c>
       <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>17:52:25</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>93</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7643,7 +7793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7656,14 +7806,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:33:57</t>
+          <t>Última actualización: 17:52:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -8572,7 +8722,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8586,7 +8736,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>97</v>
+        <v>53</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -8616,6 +8766,56 @@
       <c r="E42" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>17:52:25</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>83</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>17:52:25</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>115</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4342
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E253"/>
+  <dimension ref="A1:E254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:52:26</t>
+          <t>Última actualización: 18:08:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 248</t>
+          <t>Total filas: 249</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6037,7 +6037,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6073,7 +6073,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -6087,7 +6087,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6137,7 +6137,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6212,7 +6212,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -6237,7 +6237,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,7 +6248,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -6262,7 +6262,7 @@
         </is>
       </c>
       <c r="D237" t="n">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -6312,7 +6312,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,7 +6323,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -6337,7 +6337,7 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6373,7 +6373,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -6387,7 +6387,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6423,7 +6423,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>98</v>
+        <v>63</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -6487,7 +6487,7 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,7 +6498,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -6512,7 +6512,7 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -6537,7 +6537,7 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>110</v>
+        <v>75</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,7 +6548,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -6562,7 +6562,7 @@
         </is>
       </c>
       <c r="D249" t="n">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6623,12 +6623,12 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:48</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -6637,7 +6637,7 @@
         </is>
       </c>
       <c r="D252" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6653,18 +6653,43 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>117</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>18:08:52</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
           <t>19:50</t>
         </is>
       </c>
-      <c r="C253" t="inlineStr">
+      <c r="C254" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D253" t="n">
-        <v>118</v>
-      </c>
-      <c r="E253" t="inlineStr">
+      <c r="D254" t="n">
+        <v>102</v>
+      </c>
+      <c r="E254" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6694,7 +6719,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:52:26</t>
+          <t>Última actualización: 18:08:52</t>
         </is>
       </c>
     </row>
@@ -7635,7 +7660,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7649,7 +7674,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -7685,7 +7710,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7699,7 +7724,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -7735,7 +7760,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7749,7 +7774,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -7793,7 +7818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7806,14 +7831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:52:26</t>
+          <t>Última actualización: 18:08:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -8697,7 +8722,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -8711,7 +8736,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -8747,7 +8772,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8761,7 +8786,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>101</v>
+        <v>66</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8797,23 +8822,48 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>18:08:52</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>98</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>17:52:25</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>19:47</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D44" t="n">
+      <c r="D45" t="n">
         <v>115</v>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4343
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E254"/>
+  <dimension ref="A1:E258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:08:52</t>
+          <t>Última actualización: 18:31:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 249</t>
+          <t>Total filas: 253</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6212,7 +6212,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -6237,7 +6237,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6273,7 +6273,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -6287,7 +6287,7 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -6312,7 +6312,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6348,7 +6348,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -6362,7 +6362,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6398,7 +6398,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>17:08:17</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -6412,7 +6412,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>117</v>
+        <v>34</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,7 +6423,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -6487,7 +6487,7 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6523,21 +6523,21 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6553,16 +6553,16 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -6583,11 +6583,11 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,21 +6598,21 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>93</v>
+        <v>53</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>19:48</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>100</v>
+        <v>54</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,12 +6648,12 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:08:52</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:48</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -6662,7 +6662,7 @@
         </is>
       </c>
       <c r="D253" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,23 +6673,123 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>78</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>18:31:18</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
           <t>19:50</t>
         </is>
       </c>
-      <c r="C254" t="inlineStr">
+      <c r="C255" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D254" t="n">
-        <v>102</v>
-      </c>
-      <c r="E254" t="inlineStr">
+      <c r="D255" t="n">
+        <v>79</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>18:31:18</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>20:06</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>95</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>18:31:18</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>104</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>18:31:18</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>105</v>
+      </c>
+      <c r="E258" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6706,7 +6806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6719,14 +6819,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:08:52</t>
+          <t>Última actualización: 18:31:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 42</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -7735,7 +7835,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7749,7 +7849,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -7785,7 +7885,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -7799,9 +7899,34 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>93</v>
+        <v>54</v>
       </c>
       <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>18:31:18</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>104</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7831,7 +7956,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:08:52</t>
+          <t>Última actualización: 18:31:18</t>
         </is>
       </c>
     </row>
@@ -8747,7 +8872,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8761,7 +8886,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -8797,7 +8922,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -8811,7 +8936,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>83</v>
+        <v>44</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -8847,7 +8972,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8861,7 +8986,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>115</v>
+        <v>76</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4344
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E258"/>
+  <dimension ref="A1:E265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:31:18</t>
+          <t>Última actualización: 18:49:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 253</t>
+          <t>Total filas: 260</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -883,11 +883,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>22</v>
+        <v>95</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -6298,12 +6298,12 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:49</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -6312,7 +6312,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>18:59</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,12 +6348,12 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:59</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -6362,7 +6362,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,12 +6398,12 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -6412,7 +6412,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6428,16 +6428,16 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,12 +6448,12 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>17:52:25</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>19:13</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -6462,7 +6462,7 @@
         </is>
       </c>
       <c r="D245" t="n">
-        <v>81</v>
+        <v>22</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>17:52:25</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:13</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,7 +6498,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -6512,7 +6512,7 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>68</v>
+        <v>27</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,21 +6523,21 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,21 +6548,21 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,7 +6598,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -6608,11 +6608,11 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6628,16 +6628,16 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>19:48</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>100</v>
+        <v>54</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,12 +6673,12 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:48</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -6687,7 +6687,7 @@
         </is>
       </c>
       <c r="D254" t="n">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6703,16 +6703,16 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,21 +6723,21 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,21 +6748,21 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>104</v>
+        <v>67</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,23 +6773,198 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
+          <t>18:49:53</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>76</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
           <t>18:31:18</t>
         </is>
       </c>
-      <c r="B258" t="inlineStr">
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>20:06</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>95</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>18:49:53</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>85</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>18:49:53</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>86</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>18:31:18</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>104</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>18:31:18</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
         <is>
           <t>20:16</t>
         </is>
       </c>
-      <c r="C258" t="inlineStr">
+      <c r="C263" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D258" t="n">
+      <c r="D263" t="n">
         <v>105</v>
       </c>
-      <c r="E258" t="inlineStr">
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>18:49:53</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>110</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>18:49:53</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>112</v>
+      </c>
+      <c r="E265" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6806,7 +6981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6819,14 +6994,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:31:18</t>
+          <t>Última actualización: 18:49:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -7810,7 +7985,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7824,7 +7999,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -7860,7 +8035,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7874,7 +8049,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>76</v>
+        <v>35</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -7910,23 +8085,98 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>18:49:53</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>85</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>18:31:18</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>20:15</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D48" t="n">
+      <c r="D49" t="n">
         <v>104</v>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>18:49:53</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>110</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>18:49:53</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>112</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7943,7 +8193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7956,14 +8206,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:31:18</t>
+          <t>Última actualización: 18:49:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -8897,7 +9147,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8911,7 +9161,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>66</v>
+        <v>25</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8947,7 +9197,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:08:52</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8961,7 +9211,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>98</v>
+        <v>57</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8989,6 +9239,31 @@
         <v>76</v>
       </c>
       <c r="E45" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>18:49:53</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>20:38</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>109</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4345
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E265"/>
+  <dimension ref="A1:E268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:49:53</t>
+          <t>Última actualización: 18:59:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 260</t>
+          <t>Total filas: 263</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4183,11 +4183,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -6373,7 +6373,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -6387,7 +6387,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6423,7 +6423,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,7 +6448,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -6462,7 +6462,7 @@
         </is>
       </c>
       <c r="D245" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6498,7 +6498,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -6508,11 +6508,11 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6548,7 +6548,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -6562,7 +6562,7 @@
         </is>
       </c>
       <c r="D249" t="n">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6637,7 +6637,7 @@
         </is>
       </c>
       <c r="D252" t="n">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6662,7 +6662,7 @@
         </is>
       </c>
       <c r="D253" t="n">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6698,7 +6698,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6712,7 +6712,7 @@
         </is>
       </c>
       <c r="D255" t="n">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6737,7 +6737,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,7 +6748,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -6762,7 +6762,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,12 +6773,12 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -6787,7 +6787,7 @@
         </is>
       </c>
       <c r="D258" t="n">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,12 +6798,12 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -6812,7 +6812,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,21 +6823,21 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6853,16 +6853,16 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6887,7 +6887,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>104</v>
+        <v>76</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,12 +6898,12 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -6912,7 +6912,7 @@
         </is>
       </c>
       <c r="D263" t="n">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,21 +6923,21 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>110</v>
+        <v>77</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6953,18 +6953,93 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>110</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>18:59:14</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>101</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>18:59:14</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C265" t="inlineStr">
+      <c r="C267" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D265" t="n">
-        <v>112</v>
-      </c>
-      <c r="E265" t="inlineStr">
+      <c r="D267" t="n">
+        <v>102</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>18:59:14</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>118</v>
+      </c>
+      <c r="E268" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6981,7 +7056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6994,14 +7069,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:49:53</t>
+          <t>Última actualización: 18:59:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 46</t>
+          <t>Total filas: 47</t>
         </is>
       </c>
     </row>
@@ -8010,7 +8085,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8024,7 +8099,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -8060,7 +8135,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8074,7 +8149,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -8110,7 +8185,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -8124,7 +8199,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>104</v>
+        <v>76</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -8160,23 +8235,48 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>101</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>18:59:14</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D51" t="n">
-        <v>112</v>
-      </c>
-      <c r="E51" t="inlineStr">
+      <c r="D52" t="n">
+        <v>102</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8193,7 +8293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8206,14 +8306,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:49:53</t>
+          <t>Última actualización: 18:59:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -9172,7 +9272,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -9186,7 +9286,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -9222,7 +9322,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -9236,7 +9336,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -9264,6 +9364,31 @@
         <v>109</v>
       </c>
       <c r="E46" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>18:59:14</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>100</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4346
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E268"/>
+  <dimension ref="A1:E273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:59:15</t>
+          <t>Última actualización: 19:18:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 263</t>
+          <t>Total filas: 268</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4183,11 +4183,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6603,16 +6603,16 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,21 +6673,21 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>19:48</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>59</v>
+        <v>26</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,12 +6698,12 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:48</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -6712,7 +6712,7 @@
         </is>
       </c>
       <c r="D255" t="n">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,21 +6723,21 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,21 +6748,21 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>19:56</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>57</v>
+        <v>32</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,12 +6798,12 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -6812,7 +6812,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>76</v>
+        <v>43</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,12 +6823,12 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -6837,7 +6837,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,21 +6848,21 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,12 +6873,12 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -6887,7 +6887,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -6908,11 +6908,11 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,12 +6923,12 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -6937,7 +6937,7 @@
         </is>
       </c>
       <c r="D264" t="n">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,21 +6948,21 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>110</v>
+        <v>77</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,12 +6973,12 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -6987,7 +6987,7 @@
         </is>
       </c>
       <c r="D266" t="n">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -7003,16 +7003,16 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,23 +7023,148 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
+          <t>19:18:48</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>83</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>19:18:48</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>93</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>19:18:48</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>98</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
           <t>18:59:14</t>
         </is>
       </c>
-      <c r="B268" t="inlineStr">
+      <c r="B271" t="inlineStr">
         <is>
           <t>20:57</t>
         </is>
       </c>
-      <c r="C268" t="inlineStr">
+      <c r="C271" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D268" t="n">
+      <c r="D271" t="n">
         <v>118</v>
       </c>
-      <c r="E268" t="inlineStr">
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>19:18:48</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>107</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>19:18:48</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>108</v>
+      </c>
+      <c r="E273" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7056,7 +7181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7069,14 +7194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:59:15</t>
+          <t>Última actualización: 19:18:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 47</t>
+          <t>Total filas: 48</t>
         </is>
       </c>
     </row>
@@ -8110,7 +8235,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8124,7 +8249,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -8160,7 +8285,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -8174,7 +8299,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>85</v>
+        <v>56</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -8210,7 +8335,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -8224,7 +8349,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>110</v>
+        <v>81</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -8260,7 +8385,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -8274,9 +8399,34 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>19:18:48</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>108</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8293,7 +8443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8306,14 +8456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:59:15</t>
+          <t>Última actualización: 19:18:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 42</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -9297,37 +9447,37 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:46</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -9336,7 +9486,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -9347,12 +9497,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>20:38</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -9361,7 +9511,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>109</v>
+        <v>48</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -9372,23 +9522,48 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>19:18:48</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>20:38</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>80</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>18:59:14</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>20:39</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D47" t="n">
+      <c r="D48" t="n">
         <v>100</v>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4347
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E273"/>
+  <dimension ref="A1:E278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:18:48</t>
+          <t>Última actualización: 19:39:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 268</t>
+          <t>Total filas: 273</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D253" t="n">
@@ -6723,7 +6723,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6737,7 +6737,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,7 +6748,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -6762,7 +6762,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,7 +6773,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -6787,7 +6787,7 @@
         </is>
       </c>
       <c r="D258" t="n">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6823,12 +6823,12 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>20:04</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -6837,7 +6837,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>76</v>
+        <v>25</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,12 +6848,12 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>18:31:18</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -6862,7 +6862,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,21 +6873,21 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>18:31:18</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,12 +6898,12 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -6912,7 +6912,7 @@
         </is>
       </c>
       <c r="D263" t="n">
-        <v>76</v>
+        <v>35</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6933,11 +6933,11 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,12 +6948,12 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -6962,7 +6962,7 @@
         </is>
       </c>
       <c r="D265" t="n">
-        <v>77</v>
+        <v>36</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,21 +6998,21 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>101</v>
+        <v>57</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,21 +7023,21 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,21 +7048,21 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,21 +7073,21 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>98</v>
+        <v>62</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,21 +7098,21 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,21 +7123,21 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:54</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>107</v>
+        <v>75</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,23 +7148,148 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>77</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>18:59:14</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>118</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>19:39:42</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>86</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>19:39:42</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
           <t>21:06</t>
         </is>
       </c>
-      <c r="C273" t="inlineStr">
+      <c r="C276" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D273" t="n">
-        <v>108</v>
-      </c>
-      <c r="E273" t="inlineStr">
+      <c r="D276" t="n">
+        <v>87</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>19:39:42</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>115</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>19:39:42</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>117</v>
+      </c>
+      <c r="E278" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7194,7 +7319,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:18:48</t>
+          <t>Última actualización: 19:39:42</t>
         </is>
       </c>
     </row>
@@ -8285,7 +8410,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -8299,7 +8424,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -8335,7 +8460,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -8349,7 +8474,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -8385,7 +8510,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -8399,7 +8524,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -8410,7 +8535,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -8424,7 +8549,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -8443,7 +8568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8456,14 +8581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:18:48</t>
+          <t>Última actualización: 19:39:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -9472,7 +9597,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -9486,7 +9611,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -9564,6 +9689,31 @@
         <v>100</v>
       </c>
       <c r="E48" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>19:39:42</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>20:46</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>67</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4348
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E278"/>
+  <dimension ref="A1:E283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:39:42</t>
+          <t>Última actualización: 19:54:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 273</t>
+          <t>Total filas: 278</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -883,11 +883,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>22</v>
+        <v>95</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -6498,7 +6498,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -6508,11 +6508,11 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -6533,11 +6533,11 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:54:08</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6937,7 +6937,7 @@
         </is>
       </c>
       <c r="D264" t="n">
-        <v>76</v>
+        <v>21</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6973,7 +6973,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:54:08</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -6987,7 +6987,7 @@
         </is>
       </c>
       <c r="D266" t="n">
-        <v>77</v>
+        <v>22</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,21 +6998,21 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>19:54:08</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:19</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,21 +7023,21 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>19:54:08</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,12 +7048,12 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -7062,7 +7062,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>101</v>
+        <v>60</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,21 +7073,21 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>19:54:08</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,21 +7098,21 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>19:54:08</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>93</v>
+        <v>47</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,12 +7123,12 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>19:18:48</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>20:54</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -7137,7 +7137,7 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7153,16 +7153,16 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:54</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,21 +7173,21 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:54:08</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>118</v>
+        <v>61</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7203,16 +7203,16 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,21 +7223,21 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>19:54:08</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7253,16 +7253,16 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,23 +7273,148 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
+          <t>19:54:08</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>72</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>19:54:08</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>72</v>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>19:54:08</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>100</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>19:54:08</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>102</v>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
           <t>19:39:42</t>
         </is>
       </c>
-      <c r="B278" t="inlineStr">
+      <c r="B282" t="inlineStr">
         <is>
           <t>21:36</t>
         </is>
       </c>
-      <c r="C278" t="inlineStr">
+      <c r="C282" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D278" t="n">
+      <c r="D282" t="n">
         <v>117</v>
       </c>
-      <c r="E278" t="inlineStr">
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>19:54:08</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>103</v>
+      </c>
+      <c r="E283" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7319,7 +7444,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:39:42</t>
+          <t>Última actualización: 19:54:08</t>
         </is>
       </c>
     </row>
@@ -8435,7 +8560,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:54:08</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -8449,7 +8574,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>76</v>
+        <v>21</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -8485,7 +8610,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>19:54:08</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -8499,7 +8624,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>101</v>
+        <v>46</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -8510,7 +8635,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>19:54:08</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -8524,7 +8649,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -8535,7 +8660,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>19:54:08</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -8549,7 +8674,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -8568,7 +8693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8581,14 +8706,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:39:42</t>
+          <t>Última actualización: 19:54:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -9697,23 +9822,73 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>19:54:08</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>48</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>19:39:42</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>20:46</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D49" t="n">
+      <c r="D50" t="n">
         <v>67</v>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>19:54:08</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>98</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4349
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E283"/>
+  <dimension ref="A1:E286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:54:08</t>
+          <t>Última actualización: 20:08:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 278</t>
+          <t>Total filas: 281</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>22</v>
+        <v>95</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4183,11 +4183,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6937,7 +6937,7 @@
         </is>
       </c>
       <c r="D264" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,7 +6948,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -6962,7 +6962,7 @@
         </is>
       </c>
       <c r="D265" t="n">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -7023,21 +7023,21 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:34</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,21 +7048,21 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,12 +7073,12 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -7087,7 +7087,7 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7103,16 +7103,16 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,21 +7123,21 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>19:18:48</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>93</v>
+        <v>33</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,12 +7148,12 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>20:54</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -7162,7 +7162,7 @@
         </is>
       </c>
       <c r="D273" t="n">
-        <v>75</v>
+        <v>43</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,12 +7173,12 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:54</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -7187,7 +7187,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,21 +7198,21 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>19:54:08</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,12 +7223,12 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -7237,7 +7237,7 @@
         </is>
       </c>
       <c r="D276" t="n">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>19:54:08</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7308,11 +7308,11 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7328,16 +7328,16 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,7 +7373,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -7383,11 +7383,11 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>117</v>
+        <v>88</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,23 +7398,98 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>117</v>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>20:08:35</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
           <t>21:37</t>
         </is>
       </c>
-      <c r="C283" t="inlineStr">
+      <c r="C284" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D283" t="n">
-        <v>103</v>
-      </c>
-      <c r="E283" t="inlineStr">
+      <c r="D284" t="n">
+        <v>89</v>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>20:08:35</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>111</v>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>20:08:35</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>119</v>
+      </c>
+      <c r="E286" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7444,7 +7519,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:54:08</t>
+          <t>Última actualización: 20:08:35</t>
         </is>
       </c>
     </row>
@@ -8560,7 +8635,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -8574,7 +8649,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -8585,7 +8660,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -8599,7 +8674,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -8635,7 +8710,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -8649,7 +8724,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -8660,7 +8735,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -8674,7 +8749,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -8693,7 +8768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8706,14 +8781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:54:08</t>
+          <t>Última actualización: 20:08:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 46</t>
+          <t>Total filas: 48</t>
         </is>
       </c>
     </row>
@@ -9847,12 +9922,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>20:46</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -9861,7 +9936,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -9872,23 +9947,73 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>19:39:42</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>20:46</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>67</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>20:08:35</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>83</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>19:54:08</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>21:32</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D51" t="n">
+      <c r="D53" t="n">
         <v>98</v>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4350
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E286"/>
+  <dimension ref="A1:E290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:08:35</t>
+          <t>Última actualización: 20:30:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 281</t>
+          <t>Total filas: 285</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>22</v>
+        <v>95</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4183,11 +4183,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -6498,7 +6498,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -6508,11 +6508,11 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -6533,11 +6533,11 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -7048,7 +7048,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -7062,7 +7062,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,7 +7073,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -7087,7 +7087,7 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7137,7 +7137,7 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7162,7 +7162,7 @@
         </is>
       </c>
       <c r="D273" t="n">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7198,7 +7198,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -7212,7 +7212,7 @@
         </is>
       </c>
       <c r="D275" t="n">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,7 +7223,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -7237,7 +7237,7 @@
         </is>
       </c>
       <c r="D276" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7273,7 +7273,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -7287,7 +7287,7 @@
         </is>
       </c>
       <c r="D278" t="n">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="D279" t="n">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7362,7 +7362,7 @@
         </is>
       </c>
       <c r="D281" t="n">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,12 +7373,12 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:35</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -7387,7 +7387,7 @@
         </is>
       </c>
       <c r="D282" t="n">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,7 +7398,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>20:08:35</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -7408,11 +7408,11 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>117</v>
+        <v>88</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,12 +7423,12 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -7437,7 +7437,7 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7453,16 +7453,16 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>21:59</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,23 +7473,123 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
+          <t>20:30:47</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>88</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
           <t>20:08:35</t>
         </is>
       </c>
-      <c r="B286" t="inlineStr">
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>111</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>20:30:47</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>22:06</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>96</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>20:08:35</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
         <is>
           <t>22:07</t>
         </is>
       </c>
-      <c r="C286" t="inlineStr">
+      <c r="C289" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D286" t="n">
+      <c r="D289" t="n">
         <v>119</v>
       </c>
-      <c r="E286" t="inlineStr">
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>20:30:47</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>116</v>
+      </c>
+      <c r="E290" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7519,7 +7619,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:08:35</t>
+          <t>Última actualización: 20:30:47</t>
         </is>
       </c>
     </row>
@@ -8660,7 +8760,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -8674,7 +8774,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -8710,7 +8810,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -8724,7 +8824,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -8735,7 +8835,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -8749,7 +8849,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -8768,7 +8868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8781,14 +8881,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:08:35</t>
+          <t>Última actualización: 20:30:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 48</t>
+          <t>Total filas: 51</t>
         </is>
       </c>
     </row>
@@ -9947,12 +10047,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>19:39:42</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>20:46</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -9961,7 +10061,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>67</v>
+        <v>15</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -9972,12 +10072,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>19:39:42</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>21:31</t>
+          <t>20:46</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -9986,7 +10086,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>83</v>
+        <v>67</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -9997,25 +10097,100 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>20:08:35</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>83</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>19:54:08</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>21:32</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D53" t="n">
+      <c r="D54" t="n">
         <v>98</v>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>20:30:47</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>21:33</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>63</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>20:30:47</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>22:08</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>98</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4351
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E290"/>
+  <dimension ref="A1:E293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:30:47</t>
+          <t>Última actualización: 20:50:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 285</t>
+          <t>Total filas: 288</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -6498,7 +6498,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>18:59:14</t>
+          <t>18:49:53</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -6508,11 +6508,11 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>18:49:53</t>
+          <t>18:59:14</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -6533,11 +6533,11 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>20:30:47</t>
+          <t>20:50:08</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7162,7 +7162,7 @@
         </is>
       </c>
       <c r="D273" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7248,7 +7248,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>20:50:08</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
@@ -7262,7 +7262,7 @@
         </is>
       </c>
       <c r="D277" t="n">
-        <v>63</v>
+        <v>7</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>20:30:47</t>
+          <t>20:50:08</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="D279" t="n">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>19:54:08</t>
+          <t>20:50:08</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7337,7 +7337,7 @@
         </is>
       </c>
       <c r="D280" t="n">
-        <v>72</v>
+        <v>16</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>20:30:47</t>
+          <t>20:50:08</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:15</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>64</v>
+        <v>25</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,21 +7373,21 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>20:30:47</t>
+          <t>20:50:08</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>21:35</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>65</v>
+        <v>44</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,12 +7398,12 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:35</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -7412,7 +7412,7 @@
         </is>
       </c>
       <c r="D283" t="n">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7448,21 +7448,21 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:50:08</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>89</v>
+        <v>46</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,21 +7473,21 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>20:30:47</t>
+          <t>20:50:08</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>21:58</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>88</v>
+        <v>47</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,12 +7498,12 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>21:59</t>
+          <t>21:58</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -7512,7 +7512,7 @@
         </is>
       </c>
       <c r="D287" t="n">
-        <v>111</v>
+        <v>88</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>20:30:47</t>
+          <t>20:50:08</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>22:06</t>
+          <t>21:59</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,12 +7548,12 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>20:08:35</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>22:07</t>
+          <t>22:06</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -7562,7 +7562,7 @@
         </is>
       </c>
       <c r="D289" t="n">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,23 +7573,98 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>20:30:47</t>
+          <t>20:50:08</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>77</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>20:50:08</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
           <t>22:26</t>
         </is>
       </c>
-      <c r="C290" t="inlineStr">
+      <c r="C291" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D290" t="n">
-        <v>116</v>
-      </c>
-      <c r="E290" t="inlineStr">
+      <c r="D291" t="n">
+        <v>96</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>20:50:08</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>107</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>20:50:08</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>22:41</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>111</v>
+      </c>
+      <c r="E293" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7606,7 +7681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7619,14 +7694,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:30:47</t>
+          <t>Última actualización: 20:50:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 48</t>
+          <t>Total filas: 49</t>
         </is>
       </c>
     </row>
@@ -8835,7 +8910,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>20:30:47</t>
+          <t>20:50:08</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -8849,9 +8924,34 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>20:50:08</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>107</v>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8868,7 +8968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8881,14 +8981,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:30:47</t>
+          <t>Última actualización: 20:50:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 51</t>
+          <t>Total filas: 53</t>
         </is>
       </c>
     </row>
@@ -10172,23 +10272,73 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>20:50:08</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>44</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>20:30:47</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>22:08</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D56" t="n">
+      <c r="D57" t="n">
         <v>98</v>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>20:50:08</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>79</v>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4352
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E293"/>
+  <dimension ref="A1:E297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:50:08</t>
+          <t>Última actualización: 20:59:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 288</t>
+          <t>Total filas: 292</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>20:30:47</t>
+          <t>20:59:07</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,21 +7298,21 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>20:50:08</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>20:50:08</t>
+          <t>20:59:07</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7333,11 +7333,11 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>20:50:08</t>
+          <t>20:59:07</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>21:15</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7378,16 +7378,16 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:15</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>20:30:47</t>
+          <t>20:59:07</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>21:35</t>
+          <t>21:25</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>20:30:47</t>
+          <t>20:59:07</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,12 +7448,12 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>20:50:08</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:35</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -7462,7 +7462,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,12 +7473,12 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>20:50:08</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -7487,7 +7487,7 @@
         </is>
       </c>
       <c r="D286" t="n">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,21 +7498,21 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>20:30:47</t>
+          <t>20:59:07</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>21:58</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>88</v>
+        <v>37</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>20:50:08</t>
+          <t>20:59:07</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>21:59</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7553,16 +7553,16 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>22:06</t>
+          <t>21:58</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>20:50:08</t>
+          <t>20:59:07</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>22:07</t>
+          <t>21:59</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,17 +7598,17 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>20:50:08</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>22:26</t>
+          <t>22:06</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -7623,21 +7623,21 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>20:50:08</t>
+          <t>20:59:07</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>22:37</t>
+          <t>22:07</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>107</v>
+        <v>68</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,23 +7648,123 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>20:50:08</t>
+          <t>20:59:07</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>87</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>20:59:07</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>98</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>20:59:07</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
           <t>22:41</t>
         </is>
       </c>
-      <c r="C293" t="inlineStr">
+      <c r="C295" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D293" t="n">
-        <v>111</v>
-      </c>
-      <c r="E293" t="inlineStr">
+      <c r="D295" t="n">
+        <v>102</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>20:59:07</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>22:44</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>105</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>20:59:07</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>22:56</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>117</v>
+      </c>
+      <c r="E297" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7694,7 +7794,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:50:08</t>
+          <t>Última actualización: 20:59:07</t>
         </is>
       </c>
     </row>
@@ -8910,7 +9010,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>20:50:08</t>
+          <t>20:59:07</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -8924,7 +9024,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -8935,7 +9035,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>20:50:08</t>
+          <t>20:59:07</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -8949,7 +9049,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -8968,7 +9068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8981,14 +9081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:50:08</t>
+          <t>Última actualización: 20:59:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 53</t>
+          <t>Total filas: 54</t>
         </is>
       </c>
     </row>
@@ -10297,48 +10397,73 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>20:30:47</t>
+          <t>20:59:07</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>22:08</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-40 Y 115</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>20:50:08</t>
+          <t>20:30:47</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
+          <t>22:08</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>98</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>20:59:07</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
           <t>22:09</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D58" t="n">
-        <v>79</v>
-      </c>
-      <c r="E58" t="inlineStr">
+      <c r="D59" t="n">
+        <v>70</v>
+      </c>
+      <c r="E59" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4353
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E297"/>
+  <dimension ref="A1:E307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:59:07</t>
+          <t>Última actualización: 22:08:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 292</t>
+          <t>Total filas: 302</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:00:16</t>
+          <t>12:33:16</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>12:33:16</t>
+          <t>14:00:16</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -7648,21 +7648,21 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>20:59:07</t>
+          <t>22:08:45</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>22:26</t>
+          <t>22:08</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,21 +7673,21 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>20:59:07</t>
+          <t>22:08:45</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>22:37</t>
+          <t>22:10</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>98</v>
+        <v>2</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7703,16 +7703,16 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>22:41</t>
+          <t>22:26</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,12 +7723,12 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>20:59:07</t>
+          <t>22:08:45</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>22:44</t>
+          <t>22:33</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -7737,7 +7737,7 @@
         </is>
       </c>
       <c r="D296" t="n">
-        <v>105</v>
+        <v>25</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,23 +7748,273 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
+          <t>22:08:45</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>22:36</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>28</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
           <t>20:59:07</t>
         </is>
       </c>
-      <c r="B297" t="inlineStr">
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>98</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>22:08:45</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>22:40</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>32</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>20:59:07</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>22:41</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>102</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>20:59:07</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>22:44</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>105</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>22:08:45</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
         <is>
           <t>22:56</t>
         </is>
       </c>
-      <c r="C297" t="inlineStr">
+      <c r="C302" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D297" t="n">
-        <v>117</v>
-      </c>
-      <c r="E297" t="inlineStr">
+      <c r="D302" t="n">
+        <v>48</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>22:08:45</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>23:06</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>58</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>22:08:45</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>23:28</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>80</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>22:08:45</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>92</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>22:08:45</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>23:41</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>93</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>22:08:45</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>23:53</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>105</v>
+      </c>
+      <c r="E307" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7781,7 +8031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7794,14 +8044,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:59:07</t>
+          <t>Última actualización: 22:08:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 49</t>
+          <t>Total filas: 52</t>
         </is>
       </c>
     </row>
@@ -9035,23 +9285,98 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>22:08:45</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>22:36</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>28</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>20:59:07</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>22:37</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D54" t="n">
+      <c r="D55" t="n">
         <v>98</v>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>22:08:45</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>23:28</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>80</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>22:08:45</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>92</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9081,7 +9406,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:59:07</t>
+          <t>Última actualización: 22:08:45</t>
         </is>
       </c>
     </row>
@@ -10422,7 +10747,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>20:30:47</t>
+          <t>22:08:45</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -10436,7 +10761,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4354
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-16.xlsx
+++ b/data/horarios-141-2026-08-16.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E307"/>
+  <dimension ref="A1:E309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 22:08:45</t>
+          <t>Última actualización: 23:32:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 302</t>
+          <t>Total filas: 304</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:10:45</t>
+          <t>06:53:53</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:53:53</t>
+          <t>07:10:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>11:13:14</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>11:13:14</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>13:10:37</t>
+          <t>12:10:01</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:10:01</t>
+          <t>13:10:37</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:27:50</t>
+          <t>17:33:57</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>17:33:57</t>
+          <t>16:27:50</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>22:08:45</t>
+          <t>23:32:36</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7962,7 +7962,7 @@
         </is>
       </c>
       <c r="D305" t="n">
-        <v>92</v>
+        <v>8</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7998,23 +7998,73 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
+          <t>23:32:36</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>23:46</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>14</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
           <t>22:08:45</t>
         </is>
       </c>
-      <c r="B307" t="inlineStr">
+      <c r="B308" t="inlineStr">
         <is>
           <t>23:53</t>
         </is>
       </c>
-      <c r="C307" t="inlineStr">
+      <c r="C308" t="inlineStr">
         <is>
           <t>23_HERNANDEZ</t>
         </is>
       </c>
-      <c r="D307" t="n">
+      <c r="D308" t="n">
         <v>105</v>
       </c>
-      <c r="E307" t="inlineStr">
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>23:32:36</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>23:56</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>24</v>
+      </c>
+      <c r="E309" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8044,7 +8094,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 22:08:45</t>
+          <t>Última actualización: 23:32:36</t>
         </is>
       </c>
     </row>
@@ -9360,7 +9410,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>22:08:45</t>
+          <t>23:32:36</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -9374,7 +9424,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>92</v>
+        <v>8</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -9406,7 +9456,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 22:08:45</t>
+          <t>Última actualización: 23:32:36</t>
         </is>
       </c>
     </row>

</xml_diff>